<commit_message>
Updated cost analysis spreadsheet.
</commit_message>
<xml_diff>
--- a/Excel/Cost and CO2 analysis.xlsx
+++ b/Excel/Cost and CO2 analysis.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoa-my.sharepoint.com/personal/wwei275_uoa_auckland_ac_nz/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wwei275\Documents\GitHub\Alpha_Design_17\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{5ADCB15C-789A-4B10-9E93-AEA5B75C838A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{447082A1-038D-41D5-91FA-889913068D1E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FABC0E92-5A2F-4698-976C-7430E3D3B28C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F8E8E83B-9F9C-423D-B7EA-650D4FA9D87D}"/>
   </bookViews>
@@ -126,7 +126,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -141,13 +141,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -182,8 +196,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -520,49 +534,49 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD7E6F8D-4308-4D2A-878D-2A8D77E451CB}">
   <dimension ref="A1:I22"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="41.375" customWidth="1"/>
-    <col min="2" max="2" width="18.875" customWidth="1"/>
-    <col min="3" max="3" width="21.5" customWidth="1"/>
-    <col min="4" max="4" width="22.5" customWidth="1"/>
-    <col min="5" max="5" width="24.625" customWidth="1"/>
-    <col min="6" max="6" width="25.375" customWidth="1"/>
-    <col min="7" max="7" width="19.125" customWidth="1"/>
-    <col min="8" max="8" width="23.375" customWidth="1"/>
-    <col min="9" max="9" width="35.625" customWidth="1"/>
-    <col min="10" max="10" width="22.5" customWidth="1"/>
-    <col min="11" max="11" width="17.625" customWidth="1"/>
-    <col min="12" max="12" width="18.375" customWidth="1"/>
-    <col min="13" max="13" width="16.125" customWidth="1"/>
-    <col min="14" max="14" width="19.5" customWidth="1"/>
+    <col min="1" max="1" width="41.42578125" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" customWidth="1"/>
+    <col min="3" max="3" width="25.85546875" customWidth="1"/>
+    <col min="4" max="4" width="27.140625" customWidth="1"/>
+    <col min="5" max="5" width="29.5703125" customWidth="1"/>
+    <col min="6" max="6" width="29.28515625" customWidth="1"/>
+    <col min="7" max="7" width="19.140625" customWidth="1"/>
+    <col min="8" max="8" width="23.42578125" customWidth="1"/>
+    <col min="9" max="9" width="35.5703125" customWidth="1"/>
+    <col min="10" max="10" width="22.42578125" customWidth="1"/>
+    <col min="11" max="11" width="17.5703125" customWidth="1"/>
+    <col min="12" max="12" width="18.42578125" customWidth="1"/>
+    <col min="13" max="13" width="16.140625" customWidth="1"/>
+    <col min="14" max="14" width="19.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="1">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="4">
         <v>0</v>
       </c>
       <c r="B2" s="2">
@@ -573,25 +587,25 @@
         <f>($B$16*$B$14*0.25*A2)+$B$18</f>
         <v>24300</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <f>$B$22+($B$14*$B$19*0.25*A2)</f>
         <v>32050</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="3">
         <f>0.25*A2*$B$14*$B$15</f>
         <v>0</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="3">
         <f>0.25*A2*$B$14*$B$16</f>
         <v>0</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="3">
         <f>0.25*A2*$B$14*$B$19</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
-      <c r="A3" s="1">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
       <c r="B3" s="2">
@@ -602,25 +616,25 @@
         <f>($B$16*$B$14*0.25*A3)+$B$18</f>
         <v>26083.237499999999</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <f t="shared" ref="D3:D12" si="1">$B$22+($B$14*$B$19*0.25*A3)</f>
         <v>33868.135000000002</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="3">
         <f t="shared" ref="E3:E12" si="2">0.25*A3*$B$14*$B$15</f>
         <v>4827.9000000000005</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="3">
         <f t="shared" ref="F3:F12" si="3">0.25*A3*$B$14*$B$16</f>
         <v>1783.2375000000002</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="3">
         <f t="shared" ref="G3:G12" si="4">0.25*A3*$B$14*$B$19</f>
         <v>1818.1350000000002</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
-      <c r="A4" s="1">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
       <c r="B4" s="2">
@@ -631,25 +645,25 @@
         <f t="shared" ref="C4:C12" si="5">($B$16*$B$14*0.25*A4)+$B$18</f>
         <v>27866.474999999999</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <f t="shared" si="1"/>
         <v>35686.270000000004</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <f t="shared" si="2"/>
         <v>9655.8000000000011</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="3">
         <f t="shared" si="3"/>
         <v>3566.4750000000004</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="3">
         <f t="shared" si="4"/>
         <v>3636.2700000000004</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
-      <c r="A5" s="1">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
         <v>3</v>
       </c>
       <c r="B5" s="2">
@@ -660,25 +674,25 @@
         <f t="shared" si="5"/>
         <v>29649.712500000001</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <f t="shared" si="1"/>
         <v>37504.404999999999</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="3">
         <f t="shared" si="2"/>
         <v>14483.7</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="3">
         <f t="shared" si="3"/>
         <v>5349.7125000000005</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="3">
         <f t="shared" si="4"/>
         <v>5454.4050000000007</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
-      <c r="A6" s="1">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
         <v>4</v>
       </c>
       <c r="B6" s="2">
@@ -689,25 +703,25 @@
         <f t="shared" si="5"/>
         <v>31432.95</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <f t="shared" si="1"/>
         <v>39322.54</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="3">
         <f t="shared" si="2"/>
         <v>19311.600000000002</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="3">
         <f t="shared" si="3"/>
         <v>7132.9500000000007</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="3">
         <f t="shared" si="4"/>
         <v>7272.5400000000009</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
-      <c r="A7" s="1">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
         <v>5</v>
       </c>
       <c r="B7" s="2">
@@ -718,25 +732,25 @@
         <f t="shared" si="5"/>
         <v>33216.1875</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="2">
         <f t="shared" si="1"/>
         <v>41140.675000000003</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="3">
         <f t="shared" si="2"/>
         <v>24139.5</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="3">
         <f t="shared" si="3"/>
         <v>8916.1875</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="3">
         <f t="shared" si="4"/>
         <v>9090.6750000000011</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
-      <c r="A8" s="1">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
         <v>6</v>
       </c>
       <c r="B8" s="2">
@@ -747,25 +761,25 @@
         <f t="shared" si="5"/>
         <v>34999.425000000003</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="2">
         <f t="shared" si="1"/>
         <v>42958.81</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="3">
         <f t="shared" si="2"/>
         <v>28967.4</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="3">
         <f t="shared" si="3"/>
         <v>10699.425000000001</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="3">
         <f t="shared" si="4"/>
         <v>10908.810000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
-      <c r="A9" s="1">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="4">
         <v>7</v>
       </c>
       <c r="B9" s="2">
@@ -776,25 +790,25 @@
         <f t="shared" si="5"/>
         <v>36782.662500000006</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="2">
         <f t="shared" si="1"/>
         <v>44776.945</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="3">
         <f t="shared" si="2"/>
         <v>33795.300000000003</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="3">
         <f t="shared" si="3"/>
         <v>12482.6625</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="3">
         <f t="shared" si="4"/>
         <v>12726.945000000002</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
-      <c r="A10" s="1">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
         <v>8</v>
       </c>
       <c r="B10" s="2">
@@ -805,25 +819,25 @@
         <f t="shared" si="5"/>
         <v>38565.9</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="2">
         <f t="shared" si="1"/>
         <v>46595.08</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="3">
         <f t="shared" si="2"/>
         <v>38623.200000000004</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="3">
         <f t="shared" si="3"/>
         <v>14265.900000000001</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="3">
         <f t="shared" si="4"/>
         <v>14545.080000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
-      <c r="A11" s="1">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
         <v>9</v>
       </c>
       <c r="B11" s="2">
@@ -834,25 +848,25 @@
         <f t="shared" si="5"/>
         <v>40349.137499999997</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="2">
         <f t="shared" si="1"/>
         <v>48413.215000000004</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="3">
         <f t="shared" si="2"/>
         <v>43451.100000000006</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="3">
         <f t="shared" si="3"/>
         <v>16049.137500000001</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="3">
         <f t="shared" si="4"/>
         <v>16363.215000000002</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
-      <c r="A12" s="1">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
         <v>10</v>
       </c>
       <c r="B12" s="2">
@@ -863,57 +877,57 @@
         <f t="shared" si="5"/>
         <v>42132.375</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="2">
         <f t="shared" si="1"/>
         <v>50231.350000000006</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="3">
         <f t="shared" si="2"/>
         <v>48279</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="3">
         <f t="shared" si="3"/>
         <v>17832.375</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="3">
         <f t="shared" si="4"/>
         <v>18181.350000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
         <v>1</v>
       </c>
       <c r="B14" s="1">
         <f>12*5.5*50</f>
         <v>3300</v>
       </c>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1" t="s">
+      <c r="D14" s="4"/>
+      <c r="E14" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="F14" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="G14" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="H14" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="I14" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B15" s="1">
         <f>SUM(E15:H15)/1000</f>
         <v>5.8520000000000003</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E15" s="1"/>
@@ -924,15 +938,15 @@
       </c>
       <c r="I15" s="1"/>
     </row>
-    <row r="16" spans="1:9">
-      <c r="A16" s="1" t="s">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
         <v>11</v>
       </c>
       <c r="B16" s="1">
         <f>SUM(E18:H18)/1000</f>
         <v>2.1615000000000002</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E16" s="1"/>
@@ -943,15 +957,15 @@
       </c>
       <c r="I16" s="1"/>
     </row>
-    <row r="17" spans="1:9">
-      <c r="A17" s="1" t="s">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="3">
         <f>SUM(E19:H19)</f>
         <v>81</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" s="4" t="s">
         <v>25</v>
       </c>
       <c r="E17" s="1"/>
@@ -962,15 +976,15 @@
       </c>
       <c r="I17" s="1"/>
     </row>
-    <row r="18" spans="1:9">
-      <c r="A18" s="1" t="s">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B18" s="2">
         <f>B17*300</f>
         <v>24300</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" s="4" t="s">
         <v>26</v>
       </c>
       <c r="E18" s="1">
@@ -994,15 +1008,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
-      <c r="A19" s="1" t="s">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B19" s="1">
         <f>SUM(E16:I16)/1000</f>
         <v>2.2038000000000002</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E19" s="1"/>
@@ -1013,15 +1027,15 @@
       </c>
       <c r="I19" s="1"/>
     </row>
-    <row r="20" spans="1:9">
-      <c r="A20" s="1" t="s">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
         <v>16</v>
       </c>
       <c r="B20" s="1">
         <f>SUM(E19:I19)</f>
         <v>81</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" s="4" t="s">
         <v>9</v>
       </c>
       <c r="E20" s="1"/>
@@ -1032,8 +1046,8 @@
       </c>
       <c r="I20" s="1"/>
     </row>
-    <row r="21" spans="1:9">
-      <c r="A21" s="1" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
         <v>15</v>
       </c>
       <c r="B21" s="1">
@@ -1041,8 +1055,8 @@
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
-      <c r="A22" s="1" t="s">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B22" s="2">

</xml_diff>

<commit_message>
Populated values in Cost and CO2 analysis spreadsheet with values from Building A First Floor report.
</commit_message>
<xml_diff>
--- a/Excel/Cost and CO2 analysis.xlsx
+++ b/Excel/Cost and CO2 analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wwei275\Documents\GitHub\Alpha_Design_17\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pacopoon/Downloads/Alpha_Design_17/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FABC0E92-5A2F-4698-976C-7430E3D3B28C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C83AC0E-F4A0-DD4D-ADE6-42816B89814A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F8E8E83B-9F9C-423D-B7EA-650D4FA9D87D}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{F8E8E83B-9F9C-423D-B7EA-650D4FA9D87D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -534,25 +534,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD7E6F8D-4308-4D2A-878D-2A8D77E451CB}">
   <dimension ref="A1:I22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="41.42578125" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" customWidth="1"/>
-    <col min="3" max="3" width="25.85546875" customWidth="1"/>
-    <col min="4" max="4" width="27.140625" customWidth="1"/>
-    <col min="5" max="5" width="29.5703125" customWidth="1"/>
-    <col min="6" max="6" width="29.28515625" customWidth="1"/>
-    <col min="7" max="7" width="19.140625" customWidth="1"/>
-    <col min="8" max="8" width="23.42578125" customWidth="1"/>
-    <col min="9" max="9" width="35.5703125" customWidth="1"/>
-    <col min="10" max="10" width="22.42578125" customWidth="1"/>
-    <col min="11" max="11" width="17.5703125" customWidth="1"/>
-    <col min="12" max="12" width="18.42578125" customWidth="1"/>
-    <col min="13" max="13" width="16.140625" customWidth="1"/>
-    <col min="14" max="14" width="19.42578125" customWidth="1"/>
+    <col min="1" max="1" width="41.5" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="4" width="27.1640625" customWidth="1"/>
+    <col min="5" max="5" width="29.5" customWidth="1"/>
+    <col min="6" max="6" width="29.33203125" customWidth="1"/>
+    <col min="7" max="7" width="19.1640625" customWidth="1"/>
+    <col min="8" max="8" width="23.5" customWidth="1"/>
+    <col min="9" max="9" width="35.5" customWidth="1"/>
+    <col min="10" max="10" width="22.5" customWidth="1"/>
+    <col min="11" max="11" width="17.5" customWidth="1"/>
+    <col min="12" max="12" width="18.5" customWidth="1"/>
+    <col min="13" max="13" width="16.1640625" customWidth="1"/>
+    <col min="14" max="14" width="19.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -575,7 +575,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="4">
         <v>0</v>
       </c>
@@ -585,11 +585,11 @@
       </c>
       <c r="C2" s="2">
         <f>($B$16*$B$14*0.25*A2)+$B$18</f>
-        <v>24300</v>
+        <v>50100</v>
       </c>
       <c r="D2" s="2">
         <f>$B$22+($B$14*$B$19*0.25*A2)</f>
-        <v>32050</v>
+        <v>66350</v>
       </c>
       <c r="E2" s="3">
         <f>0.25*A2*$B$14*$B$15</f>
@@ -604,297 +604,297 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="4">
         <v>1</v>
       </c>
       <c r="B3" s="2">
         <f t="shared" ref="B3:B12" si="0">$B$15*0.25*$B$14*A3</f>
-        <v>4827.9000000000005</v>
+        <v>9655.8000000000011</v>
       </c>
       <c r="C3" s="2">
         <f>($B$16*$B$14*0.25*A3)+$B$18</f>
-        <v>26083.237499999999</v>
+        <v>54242.737500000003</v>
       </c>
       <c r="D3" s="2">
         <f t="shared" ref="D3:D12" si="1">$B$22+($B$14*$B$19*0.25*A3)</f>
-        <v>33868.135000000002</v>
+        <v>70564.759999999995</v>
       </c>
       <c r="E3" s="3">
         <f t="shared" ref="E3:E12" si="2">0.25*A3*$B$14*$B$15</f>
-        <v>4827.9000000000005</v>
+        <v>9655.8000000000011</v>
       </c>
       <c r="F3" s="3">
         <f t="shared" ref="F3:F12" si="3">0.25*A3*$B$14*$B$16</f>
-        <v>1783.2375000000002</v>
+        <v>4142.7374999999993</v>
       </c>
       <c r="G3" s="3">
         <f t="shared" ref="G3:G12" si="4">0.25*A3*$B$14*$B$19</f>
-        <v>1818.1350000000002</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+        <v>4214.76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>2</v>
       </c>
       <c r="B4" s="2">
         <f t="shared" si="0"/>
-        <v>9655.8000000000011</v>
+        <v>19311.600000000002</v>
       </c>
       <c r="C4" s="2">
         <f t="shared" ref="C4:C12" si="5">($B$16*$B$14*0.25*A4)+$B$18</f>
-        <v>27866.474999999999</v>
+        <v>58385.474999999999</v>
       </c>
       <c r="D4" s="2">
         <f t="shared" si="1"/>
-        <v>35686.270000000004</v>
+        <v>74779.520000000004</v>
       </c>
       <c r="E4" s="3">
         <f t="shared" si="2"/>
-        <v>9655.8000000000011</v>
+        <v>19311.600000000002</v>
       </c>
       <c r="F4" s="3">
         <f t="shared" si="3"/>
-        <v>3566.4750000000004</v>
+        <v>8285.4749999999985</v>
       </c>
       <c r="G4" s="3">
         <f t="shared" si="4"/>
-        <v>3636.2700000000004</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+        <v>8429.52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>3</v>
       </c>
       <c r="B5" s="2">
         <f t="shared" si="0"/>
-        <v>14483.7</v>
+        <v>28967.4</v>
       </c>
       <c r="C5" s="2">
         <f t="shared" si="5"/>
-        <v>29649.712500000001</v>
+        <v>62528.212499999994</v>
       </c>
       <c r="D5" s="2">
         <f t="shared" si="1"/>
-        <v>37504.404999999999</v>
+        <v>78994.28</v>
       </c>
       <c r="E5" s="3">
         <f t="shared" si="2"/>
-        <v>14483.7</v>
+        <v>28967.4</v>
       </c>
       <c r="F5" s="3">
         <f t="shared" si="3"/>
-        <v>5349.7125000000005</v>
+        <v>12428.2125</v>
       </c>
       <c r="G5" s="3">
         <f t="shared" si="4"/>
-        <v>5454.4050000000007</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>12644.28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>4</v>
       </c>
       <c r="B6" s="2">
         <f t="shared" si="0"/>
-        <v>19311.600000000002</v>
+        <v>38623.200000000004</v>
       </c>
       <c r="C6" s="2">
         <f t="shared" si="5"/>
-        <v>31432.95</v>
+        <v>66670.95</v>
       </c>
       <c r="D6" s="2">
         <f t="shared" si="1"/>
-        <v>39322.54</v>
+        <v>83209.040000000008</v>
       </c>
       <c r="E6" s="3">
         <f t="shared" si="2"/>
-        <v>19311.600000000002</v>
+        <v>38623.200000000004</v>
       </c>
       <c r="F6" s="3">
         <f t="shared" si="3"/>
-        <v>7132.9500000000007</v>
+        <v>16570.949999999997</v>
       </c>
       <c r="G6" s="3">
         <f t="shared" si="4"/>
-        <v>7272.5400000000009</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>16859.04</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="4">
         <v>5</v>
       </c>
       <c r="B7" s="2">
         <f t="shared" si="0"/>
-        <v>24139.500000000004</v>
+        <v>48279.000000000007</v>
       </c>
       <c r="C7" s="2">
         <f t="shared" si="5"/>
-        <v>33216.1875</v>
+        <v>70813.6875</v>
       </c>
       <c r="D7" s="2">
         <f t="shared" si="1"/>
-        <v>41140.675000000003</v>
+        <v>87423.8</v>
       </c>
       <c r="E7" s="3">
         <f t="shared" si="2"/>
-        <v>24139.5</v>
+        <v>48279</v>
       </c>
       <c r="F7" s="3">
         <f t="shared" si="3"/>
-        <v>8916.1875</v>
+        <v>20713.6875</v>
       </c>
       <c r="G7" s="3">
         <f t="shared" si="4"/>
-        <v>9090.6750000000011</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+        <v>21073.800000000003</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
         <v>6</v>
       </c>
       <c r="B8" s="2">
         <f t="shared" si="0"/>
-        <v>28967.4</v>
+        <v>57934.8</v>
       </c>
       <c r="C8" s="2">
         <f t="shared" si="5"/>
-        <v>34999.425000000003</v>
+        <v>74956.424999999988</v>
       </c>
       <c r="D8" s="2">
         <f t="shared" si="1"/>
-        <v>42958.81</v>
+        <v>91638.56</v>
       </c>
       <c r="E8" s="3">
         <f t="shared" si="2"/>
-        <v>28967.4</v>
+        <v>57934.8</v>
       </c>
       <c r="F8" s="3">
         <f t="shared" si="3"/>
-        <v>10699.425000000001</v>
+        <v>24856.424999999999</v>
       </c>
       <c r="G8" s="3">
         <f t="shared" si="4"/>
-        <v>10908.810000000001</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+        <v>25288.560000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="4">
         <v>7</v>
       </c>
       <c r="B9" s="2">
         <f t="shared" si="0"/>
-        <v>33795.300000000003</v>
+        <v>67590.600000000006</v>
       </c>
       <c r="C9" s="2">
         <f t="shared" si="5"/>
-        <v>36782.662500000006</v>
+        <v>79099.162499999991</v>
       </c>
       <c r="D9" s="2">
         <f t="shared" si="1"/>
-        <v>44776.945</v>
+        <v>95853.32</v>
       </c>
       <c r="E9" s="3">
         <f t="shared" si="2"/>
-        <v>33795.300000000003</v>
+        <v>67590.600000000006</v>
       </c>
       <c r="F9" s="3">
         <f t="shared" si="3"/>
-        <v>12482.6625</v>
+        <v>28999.162499999999</v>
       </c>
       <c r="G9" s="3">
         <f t="shared" si="4"/>
-        <v>12726.945000000002</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+        <v>29503.320000000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
         <v>8</v>
       </c>
       <c r="B10" s="2">
         <f t="shared" si="0"/>
-        <v>38623.200000000004</v>
+        <v>77246.400000000009</v>
       </c>
       <c r="C10" s="2">
         <f t="shared" si="5"/>
-        <v>38565.9</v>
+        <v>83241.899999999994</v>
       </c>
       <c r="D10" s="2">
         <f t="shared" si="1"/>
-        <v>46595.08</v>
+        <v>100068.08</v>
       </c>
       <c r="E10" s="3">
         <f t="shared" si="2"/>
-        <v>38623.200000000004</v>
+        <v>77246.400000000009</v>
       </c>
       <c r="F10" s="3">
         <f t="shared" si="3"/>
-        <v>14265.900000000001</v>
+        <v>33141.899999999994</v>
       </c>
       <c r="G10" s="3">
         <f t="shared" si="4"/>
-        <v>14545.080000000002</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+        <v>33718.080000000002</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="4">
         <v>9</v>
       </c>
       <c r="B11" s="2">
         <f t="shared" si="0"/>
-        <v>43451.100000000006</v>
+        <v>86902.200000000012</v>
       </c>
       <c r="C11" s="2">
         <f t="shared" si="5"/>
-        <v>40349.137499999997</v>
+        <v>87384.637499999997</v>
       </c>
       <c r="D11" s="2">
         <f t="shared" si="1"/>
-        <v>48413.215000000004</v>
+        <v>104282.84</v>
       </c>
       <c r="E11" s="3">
         <f t="shared" si="2"/>
-        <v>43451.100000000006</v>
+        <v>86902.200000000012</v>
       </c>
       <c r="F11" s="3">
         <f t="shared" si="3"/>
-        <v>16049.137500000001</v>
+        <v>37284.637499999997</v>
       </c>
       <c r="G11" s="3">
         <f t="shared" si="4"/>
-        <v>16363.215000000002</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+        <v>37932.840000000004</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="4">
         <v>10</v>
       </c>
       <c r="B12" s="2">
         <f t="shared" si="0"/>
-        <v>48279.000000000007</v>
+        <v>96558.000000000015</v>
       </c>
       <c r="C12" s="2">
         <f t="shared" si="5"/>
-        <v>42132.375</v>
+        <v>91527.375</v>
       </c>
       <c r="D12" s="2">
         <f t="shared" si="1"/>
-        <v>50231.350000000006</v>
+        <v>108497.60000000001</v>
       </c>
       <c r="E12" s="3">
         <f t="shared" si="2"/>
-        <v>48279</v>
+        <v>96558</v>
       </c>
       <c r="F12" s="3">
         <f t="shared" si="3"/>
-        <v>17832.375</v>
+        <v>41427.375</v>
       </c>
       <c r="G12" s="3">
         <f t="shared" si="4"/>
-        <v>18181.350000000002</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+        <v>42147.600000000006</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>1</v>
       </c>
@@ -919,70 +919,76 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B15" s="1">
         <f>SUM(E15:H15)/1000</f>
-        <v>5.8520000000000003</v>
+        <v>11.704000000000001</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
+      <c r="F15" s="1">
+        <v>5852</v>
+      </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1">
         <v>5852</v>
       </c>
       <c r="I15" s="1"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>11</v>
       </c>
       <c r="B16" s="1">
         <f>SUM(E18:H18)/1000</f>
-        <v>2.1615000000000002</v>
+        <v>5.0214999999999996</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
+      <c r="F16" s="1">
+        <v>2905</v>
+      </c>
       <c r="G16" s="1"/>
       <c r="H16" s="1">
         <v>2203.8000000000002</v>
       </c>
       <c r="I16" s="1"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B17" s="3">
         <f>SUM(E19:H19)</f>
-        <v>81</v>
+        <v>167</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>25</v>
       </c>
       <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
+      <c r="F17" s="1">
+        <v>45</v>
+      </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1">
         <v>42.3</v>
       </c>
       <c r="I17" s="1"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B18" s="2">
         <f>B17*300</f>
-        <v>24300</v>
+        <v>50100</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>26</v>
@@ -992,76 +998,80 @@
         <v>0</v>
       </c>
       <c r="F18" s="1">
-        <f t="shared" ref="F18" si="6">F16-F17</f>
+        <f>F16-F17</f>
+        <v>2860</v>
+      </c>
+      <c r="G18" s="1">
+        <f t="shared" ref="G18" si="6">G16-G17</f>
         <v>0</v>
       </c>
-      <c r="G18" s="1">
-        <f t="shared" ref="G18" si="7">G16-G17</f>
+      <c r="H18" s="1">
+        <f t="shared" ref="H18" si="7">H16-H17</f>
+        <v>2161.5</v>
+      </c>
+      <c r="I18" s="1">
+        <f t="shared" ref="I18" si="8">I16-I17</f>
         <v>0</v>
       </c>
-      <c r="H18" s="1">
-        <f t="shared" ref="H18" si="8">H16-H17</f>
-        <v>2161.5</v>
-      </c>
-      <c r="I18" s="1">
-        <f t="shared" ref="I18" si="9">I16-I17</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B19" s="1">
         <f>SUM(E16:I16)/1000</f>
-        <v>2.2038000000000002</v>
+        <v>5.1088000000000005</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
+      <c r="F19" s="1">
+        <v>86</v>
+      </c>
       <c r="G19" s="1"/>
       <c r="H19" s="1">
         <v>81</v>
       </c>
       <c r="I19" s="1"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>16</v>
       </c>
       <c r="B20" s="1">
         <f>SUM(E19:I19)</f>
-        <v>81</v>
+        <v>167</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>9</v>
       </c>
       <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
+      <c r="F20" s="1">
+        <v>34</v>
+      </c>
       <c r="G20" s="1"/>
       <c r="H20" s="1">
         <v>31</v>
       </c>
       <c r="I20" s="1"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>15</v>
       </c>
       <c r="B21" s="1">
         <f>SUM(E20:I20)</f>
-        <v>31</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B22" s="2">
         <f>(B20*300)+(B21*250)</f>
-        <v>32050</v>
+        <v>66350</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Cost and C02 Analysis excel sheet for building A ground floor
</commit_message>
<xml_diff>
--- a/Excel/Cost and CO2 analysis.xlsx
+++ b/Excel/Cost and CO2 analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pacopoon/Downloads/Alpha_Design_17/Excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester1\ELECTENG310\Alpha_Design_17\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C83AC0E-F4A0-DD4D-ADE6-42816B89814A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13808E69-2BB3-4B5A-AD62-D9A4ABF80B23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{F8E8E83B-9F9C-423D-B7EA-650D4FA9D87D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F8E8E83B-9F9C-423D-B7EA-650D4FA9D87D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -124,7 +124,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -190,12 +190,12 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
@@ -534,25 +534,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD7E6F8D-4308-4D2A-878D-2A8D77E451CB}">
   <dimension ref="A1:I22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="41.5" customWidth="1"/>
+    <col min="1" max="1" width="41.44140625" customWidth="1"/>
     <col min="2" max="2" width="23.6640625" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="27.1640625" customWidth="1"/>
-    <col min="5" max="5" width="29.5" customWidth="1"/>
+    <col min="3" max="3" width="25.77734375" customWidth="1"/>
+    <col min="4" max="4" width="27.109375" customWidth="1"/>
+    <col min="5" max="5" width="29.44140625" customWidth="1"/>
     <col min="6" max="6" width="29.33203125" customWidth="1"/>
-    <col min="7" max="7" width="19.1640625" customWidth="1"/>
-    <col min="8" max="8" width="23.5" customWidth="1"/>
-    <col min="9" max="9" width="35.5" customWidth="1"/>
-    <col min="10" max="10" width="22.5" customWidth="1"/>
-    <col min="11" max="11" width="17.5" customWidth="1"/>
-    <col min="12" max="12" width="18.5" customWidth="1"/>
-    <col min="13" max="13" width="16.1640625" customWidth="1"/>
-    <col min="14" max="14" width="19.5" customWidth="1"/>
+    <col min="7" max="7" width="19.109375" customWidth="1"/>
+    <col min="8" max="8" width="23.44140625" customWidth="1"/>
+    <col min="9" max="9" width="35.44140625" customWidth="1"/>
+    <col min="10" max="10" width="22.44140625" customWidth="1"/>
+    <col min="11" max="11" width="17.44140625" customWidth="1"/>
+    <col min="12" max="12" width="18.44140625" customWidth="1"/>
+    <col min="13" max="13" width="16.109375" customWidth="1"/>
+    <col min="14" max="14" width="19.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -575,7 +575,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>0</v>
       </c>
@@ -585,11 +585,11 @@
       </c>
       <c r="C2" s="2">
         <f>($B$16*$B$14*0.25*A2)+$B$18</f>
-        <v>50100</v>
+        <v>69300</v>
       </c>
       <c r="D2" s="2">
         <f>$B$22+($B$14*$B$19*0.25*A2)</f>
-        <v>66350</v>
+        <v>93050</v>
       </c>
       <c r="E2" s="3">
         <f>0.25*A2*$B$14*$B$15</f>
@@ -604,297 +604,297 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>1</v>
       </c>
       <c r="B3" s="2">
         <f t="shared" ref="B3:B12" si="0">$B$15*0.25*$B$14*A3</f>
-        <v>9655.8000000000011</v>
+        <v>14556.3</v>
       </c>
       <c r="C3" s="2">
         <f>($B$16*$B$14*0.25*A3)+$B$18</f>
-        <v>54242.737500000003</v>
+        <v>74326.065000000002</v>
       </c>
       <c r="D3" s="2">
         <f t="shared" ref="D3:D12" si="1">$B$22+($B$14*$B$19*0.25*A3)</f>
-        <v>70564.759999999995</v>
+        <v>98172.837499999994</v>
       </c>
       <c r="E3" s="3">
         <f t="shared" ref="E3:E12" si="2">0.25*A3*$B$14*$B$15</f>
-        <v>9655.8000000000011</v>
+        <v>14556.3</v>
       </c>
       <c r="F3" s="3">
         <f t="shared" ref="F3:F12" si="3">0.25*A3*$B$14*$B$16</f>
-        <v>4142.7374999999993</v>
+        <v>5026.0649999999996</v>
       </c>
       <c r="G3" s="3">
         <f t="shared" ref="G3:G12" si="4">0.25*A3*$B$14*$B$19</f>
-        <v>4214.76</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+        <v>5122.8375000000005</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>2</v>
       </c>
       <c r="B4" s="2">
         <f t="shared" si="0"/>
-        <v>19311.600000000002</v>
+        <v>29112.6</v>
       </c>
       <c r="C4" s="2">
         <f t="shared" ref="C4:C12" si="5">($B$16*$B$14*0.25*A4)+$B$18</f>
-        <v>58385.474999999999</v>
+        <v>79352.13</v>
       </c>
       <c r="D4" s="2">
         <f t="shared" si="1"/>
-        <v>74779.520000000004</v>
+        <v>103295.675</v>
       </c>
       <c r="E4" s="3">
         <f t="shared" si="2"/>
-        <v>19311.600000000002</v>
+        <v>29112.6</v>
       </c>
       <c r="F4" s="3">
         <f t="shared" si="3"/>
-        <v>8285.4749999999985</v>
+        <v>10052.129999999999</v>
       </c>
       <c r="G4" s="3">
         <f t="shared" si="4"/>
-        <v>8429.52</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+        <v>10245.675000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>3</v>
       </c>
       <c r="B5" s="2">
         <f t="shared" si="0"/>
-        <v>28967.4</v>
+        <v>43668.899999999994</v>
       </c>
       <c r="C5" s="2">
         <f t="shared" si="5"/>
-        <v>62528.212499999994</v>
+        <v>84378.195000000007</v>
       </c>
       <c r="D5" s="2">
         <f t="shared" si="1"/>
-        <v>78994.28</v>
+        <v>108418.5125</v>
       </c>
       <c r="E5" s="3">
         <f t="shared" si="2"/>
-        <v>28967.4</v>
+        <v>43668.899999999994</v>
       </c>
       <c r="F5" s="3">
         <f t="shared" si="3"/>
-        <v>12428.2125</v>
+        <v>15078.195</v>
       </c>
       <c r="G5" s="3">
         <f t="shared" si="4"/>
-        <v>12644.28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+        <v>15368.512500000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>4</v>
       </c>
       <c r="B6" s="2">
         <f t="shared" si="0"/>
-        <v>38623.200000000004</v>
+        <v>58225.2</v>
       </c>
       <c r="C6" s="2">
         <f t="shared" si="5"/>
-        <v>66670.95</v>
+        <v>89404.26</v>
       </c>
       <c r="D6" s="2">
         <f t="shared" si="1"/>
-        <v>83209.040000000008</v>
+        <v>113541.35</v>
       </c>
       <c r="E6" s="3">
         <f t="shared" si="2"/>
-        <v>38623.200000000004</v>
+        <v>58225.2</v>
       </c>
       <c r="F6" s="3">
         <f t="shared" si="3"/>
-        <v>16570.949999999997</v>
+        <v>20104.259999999998</v>
       </c>
       <c r="G6" s="3">
         <f t="shared" si="4"/>
-        <v>16859.04</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+        <v>20491.350000000002</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>5</v>
       </c>
       <c r="B7" s="2">
         <f t="shared" si="0"/>
-        <v>48279.000000000007</v>
+        <v>72781.5</v>
       </c>
       <c r="C7" s="2">
         <f t="shared" si="5"/>
-        <v>70813.6875</v>
+        <v>94430.324999999997</v>
       </c>
       <c r="D7" s="2">
         <f t="shared" si="1"/>
-        <v>87423.8</v>
+        <v>118664.1875</v>
       </c>
       <c r="E7" s="3">
         <f t="shared" si="2"/>
-        <v>48279</v>
+        <v>72781.5</v>
       </c>
       <c r="F7" s="3">
         <f t="shared" si="3"/>
-        <v>20713.6875</v>
+        <v>25130.325000000001</v>
       </c>
       <c r="G7" s="3">
         <f t="shared" si="4"/>
-        <v>21073.800000000003</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+        <v>25614.1875</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>6</v>
       </c>
       <c r="B8" s="2">
         <f t="shared" si="0"/>
-        <v>57934.8</v>
+        <v>87337.799999999988</v>
       </c>
       <c r="C8" s="2">
         <f t="shared" si="5"/>
-        <v>74956.424999999988</v>
+        <v>99456.39</v>
       </c>
       <c r="D8" s="2">
         <f t="shared" si="1"/>
-        <v>91638.56</v>
+        <v>123787.02499999999</v>
       </c>
       <c r="E8" s="3">
         <f t="shared" si="2"/>
-        <v>57934.8</v>
+        <v>87337.799999999988</v>
       </c>
       <c r="F8" s="3">
         <f t="shared" si="3"/>
-        <v>24856.424999999999</v>
+        <v>30156.39</v>
       </c>
       <c r="G8" s="3">
         <f t="shared" si="4"/>
-        <v>25288.560000000001</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+        <v>30737.025000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>7</v>
       </c>
       <c r="B9" s="2">
         <f t="shared" si="0"/>
-        <v>67590.600000000006</v>
+        <v>101894.09999999999</v>
       </c>
       <c r="C9" s="2">
         <f t="shared" si="5"/>
-        <v>79099.162499999991</v>
+        <v>104482.45499999999</v>
       </c>
       <c r="D9" s="2">
         <f t="shared" si="1"/>
-        <v>95853.32</v>
+        <v>128909.8625</v>
       </c>
       <c r="E9" s="3">
         <f t="shared" si="2"/>
-        <v>67590.600000000006</v>
+        <v>101894.09999999999</v>
       </c>
       <c r="F9" s="3">
         <f t="shared" si="3"/>
-        <v>28999.162499999999</v>
+        <v>35182.455000000002</v>
       </c>
       <c r="G9" s="3">
         <f t="shared" si="4"/>
-        <v>29503.320000000003</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+        <v>35859.862500000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>8</v>
       </c>
       <c r="B10" s="2">
         <f t="shared" si="0"/>
-        <v>77246.400000000009</v>
+        <v>116450.4</v>
       </c>
       <c r="C10" s="2">
         <f t="shared" si="5"/>
-        <v>83241.899999999994</v>
+        <v>109508.51999999999</v>
       </c>
       <c r="D10" s="2">
         <f t="shared" si="1"/>
-        <v>100068.08</v>
+        <v>134032.70000000001</v>
       </c>
       <c r="E10" s="3">
         <f t="shared" si="2"/>
-        <v>77246.400000000009</v>
+        <v>116450.4</v>
       </c>
       <c r="F10" s="3">
         <f t="shared" si="3"/>
-        <v>33141.899999999994</v>
+        <v>40208.519999999997</v>
       </c>
       <c r="G10" s="3">
         <f t="shared" si="4"/>
-        <v>33718.080000000002</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+        <v>40982.700000000004</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>9</v>
       </c>
       <c r="B11" s="2">
         <f t="shared" si="0"/>
-        <v>86902.200000000012</v>
+        <v>131006.7</v>
       </c>
       <c r="C11" s="2">
         <f t="shared" si="5"/>
-        <v>87384.637499999997</v>
+        <v>114534.58499999999</v>
       </c>
       <c r="D11" s="2">
         <f t="shared" si="1"/>
-        <v>104282.84</v>
+        <v>139155.53750000001</v>
       </c>
       <c r="E11" s="3">
         <f t="shared" si="2"/>
-        <v>86902.200000000012</v>
+        <v>131006.69999999998</v>
       </c>
       <c r="F11" s="3">
         <f t="shared" si="3"/>
-        <v>37284.637499999997</v>
+        <v>45234.584999999999</v>
       </c>
       <c r="G11" s="3">
         <f t="shared" si="4"/>
-        <v>37932.840000000004</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+        <v>46105.537499999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>10</v>
       </c>
       <c r="B12" s="2">
         <f t="shared" si="0"/>
-        <v>96558.000000000015</v>
+        <v>145563</v>
       </c>
       <c r="C12" s="2">
         <f t="shared" si="5"/>
-        <v>91527.375</v>
+        <v>119560.65</v>
       </c>
       <c r="D12" s="2">
         <f t="shared" si="1"/>
-        <v>108497.60000000001</v>
+        <v>144278.375</v>
       </c>
       <c r="E12" s="3">
         <f t="shared" si="2"/>
-        <v>96558</v>
+        <v>145563</v>
       </c>
       <c r="F12" s="3">
         <f t="shared" si="3"/>
-        <v>41427.375</v>
+        <v>50260.65</v>
       </c>
       <c r="G12" s="3">
         <f t="shared" si="4"/>
-        <v>42147.600000000006</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+        <v>51228.375</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>1</v>
       </c>
@@ -919,18 +919,20 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B15" s="1">
         <f>SUM(E15:H15)/1000</f>
-        <v>11.704000000000001</v>
+        <v>17.643999999999998</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E15" s="1"/>
+      <c r="E15" s="1">
+        <v>5940</v>
+      </c>
       <c r="F15" s="1">
         <v>5852</v>
       </c>
@@ -940,18 +942,20 @@
       </c>
       <c r="I15" s="1"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>11</v>
       </c>
       <c r="B16" s="1">
         <f>SUM(E18:H18)/1000</f>
-        <v>5.0214999999999996</v>
+        <v>6.0922000000000001</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E16" s="1"/>
+      <c r="E16" s="1">
+        <v>1100.7</v>
+      </c>
       <c r="F16" s="1">
         <v>2905</v>
       </c>
@@ -961,18 +965,20 @@
       </c>
       <c r="I16" s="1"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B17" s="3">
         <f>SUM(E19:H19)</f>
-        <v>167</v>
+        <v>231</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E17" s="1"/>
+      <c r="E17" s="1">
+        <v>30</v>
+      </c>
       <c r="F17" s="1">
         <v>45</v>
       </c>
@@ -982,20 +988,20 @@
       </c>
       <c r="I17" s="1"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B18" s="2">
         <f>B17*300</f>
-        <v>50100</v>
+        <v>69300</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>26</v>
       </c>
       <c r="E18" s="1">
         <f>E16-E17</f>
-        <v>0</v>
+        <v>1070.7</v>
       </c>
       <c r="F18" s="1">
         <f>F16-F17</f>
@@ -1014,18 +1020,20 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B19" s="1">
         <f>SUM(E16:I16)/1000</f>
-        <v>5.1088000000000005</v>
+        <v>6.2095000000000002</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E19" s="1"/>
+      <c r="E19" s="1">
+        <v>64</v>
+      </c>
       <c r="F19" s="1">
         <v>86</v>
       </c>
@@ -1035,18 +1043,20 @@
       </c>
       <c r="I19" s="1"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>16</v>
       </c>
       <c r="B20" s="1">
         <f>SUM(E19:I19)</f>
-        <v>167</v>
+        <v>231</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="1"/>
+      <c r="E20" s="1">
+        <v>30</v>
+      </c>
       <c r="F20" s="1">
         <v>34</v>
       </c>
@@ -1056,22 +1066,22 @@
       </c>
       <c r="I20" s="1"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>15</v>
       </c>
       <c r="B21" s="1">
         <f>SUM(E20:I20)</f>
-        <v>65</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B22" s="2">
         <f>(B20*300)+(B21*250)</f>
-        <v>66350</v>
+        <v>93050</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update car park excel
</commit_message>
<xml_diff>
--- a/Excel/Cost and CO2 analysis.xlsx
+++ b/Excel/Cost and CO2 analysis.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester1\ELECTENG310\Alpha_Design_17\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\310_Project1\Alpha_Design_17\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13808E69-2BB3-4B5A-AD62-D9A4ABF80B23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FE54094-97F6-4839-AA0B-E9AF3D2B7AAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F8E8E83B-9F9C-423D-B7EA-650D4FA9D87D}"/>
   </bookViews>
@@ -589,7 +589,7 @@
       </c>
       <c r="D2" s="2">
         <f>$B$22+($B$14*$B$19*0.25*A2)</f>
-        <v>93050</v>
+        <v>144400</v>
       </c>
       <c r="E2" s="3">
         <f>0.25*A2*$B$14*$B$15</f>
@@ -618,7 +618,7 @@
       </c>
       <c r="D3" s="2">
         <f t="shared" ref="D3:D12" si="1">$B$22+($B$14*$B$19*0.25*A3)</f>
-        <v>98172.837499999994</v>
+        <v>151818.73000000001</v>
       </c>
       <c r="E3" s="3">
         <f t="shared" ref="E3:E12" si="2">0.25*A3*$B$14*$B$15</f>
@@ -630,7 +630,7 @@
       </c>
       <c r="G3" s="3">
         <f t="shared" ref="G3:G12" si="4">0.25*A3*$B$14*$B$19</f>
-        <v>5122.8375000000005</v>
+        <v>7418.73</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -647,7 +647,7 @@
       </c>
       <c r="D4" s="2">
         <f t="shared" si="1"/>
-        <v>103295.675</v>
+        <v>159237.46</v>
       </c>
       <c r="E4" s="3">
         <f t="shared" si="2"/>
@@ -659,7 +659,7 @@
       </c>
       <c r="G4" s="3">
         <f t="shared" si="4"/>
-        <v>10245.675000000001</v>
+        <v>14837.46</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -676,7 +676,7 @@
       </c>
       <c r="D5" s="2">
         <f t="shared" si="1"/>
-        <v>108418.5125</v>
+        <v>166656.19</v>
       </c>
       <c r="E5" s="3">
         <f t="shared" si="2"/>
@@ -688,7 +688,7 @@
       </c>
       <c r="G5" s="3">
         <f t="shared" si="4"/>
-        <v>15368.512500000001</v>
+        <v>22256.19</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -705,7 +705,7 @@
       </c>
       <c r="D6" s="2">
         <f t="shared" si="1"/>
-        <v>113541.35</v>
+        <v>174074.91999999998</v>
       </c>
       <c r="E6" s="3">
         <f t="shared" si="2"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="G6" s="3">
         <f t="shared" si="4"/>
-        <v>20491.350000000002</v>
+        <v>29674.92</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -734,7 +734,7 @@
       </c>
       <c r="D7" s="2">
         <f t="shared" si="1"/>
-        <v>118664.1875</v>
+        <v>181493.65</v>
       </c>
       <c r="E7" s="3">
         <f t="shared" si="2"/>
@@ -746,7 +746,7 @@
       </c>
       <c r="G7" s="3">
         <f t="shared" si="4"/>
-        <v>25614.1875</v>
+        <v>37093.65</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -763,7 +763,7 @@
       </c>
       <c r="D8" s="2">
         <f t="shared" si="1"/>
-        <v>123787.02499999999</v>
+        <v>188912.38</v>
       </c>
       <c r="E8" s="3">
         <f t="shared" si="2"/>
@@ -775,7 +775,7 @@
       </c>
       <c r="G8" s="3">
         <f t="shared" si="4"/>
-        <v>30737.025000000001</v>
+        <v>44512.38</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -792,7 +792,7 @@
       </c>
       <c r="D9" s="2">
         <f t="shared" si="1"/>
-        <v>128909.8625</v>
+        <v>196331.11</v>
       </c>
       <c r="E9" s="3">
         <f t="shared" si="2"/>
@@ -804,7 +804,7 @@
       </c>
       <c r="G9" s="3">
         <f t="shared" si="4"/>
-        <v>35859.862500000003</v>
+        <v>51931.11</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -821,7 +821,7 @@
       </c>
       <c r="D10" s="2">
         <f t="shared" si="1"/>
-        <v>134032.70000000001</v>
+        <v>203749.84</v>
       </c>
       <c r="E10" s="3">
         <f t="shared" si="2"/>
@@ -833,7 +833,7 @@
       </c>
       <c r="G10" s="3">
         <f t="shared" si="4"/>
-        <v>40982.700000000004</v>
+        <v>59349.84</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -850,7 +850,7 @@
       </c>
       <c r="D11" s="2">
         <f t="shared" si="1"/>
-        <v>139155.53750000001</v>
+        <v>211168.57</v>
       </c>
       <c r="E11" s="3">
         <f t="shared" si="2"/>
@@ -862,7 +862,7 @@
       </c>
       <c r="G11" s="3">
         <f t="shared" si="4"/>
-        <v>46105.537499999999</v>
+        <v>66768.569999999992</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -879,7 +879,7 @@
       </c>
       <c r="D12" s="2">
         <f t="shared" si="1"/>
-        <v>144278.375</v>
+        <v>218587.3</v>
       </c>
       <c r="E12" s="3">
         <f t="shared" si="2"/>
@@ -891,7 +891,7 @@
       </c>
       <c r="G12" s="3">
         <f t="shared" si="4"/>
-        <v>51228.375</v>
+        <v>74187.3</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
@@ -940,7 +940,9 @@
       <c r="H15" s="1">
         <v>5852</v>
       </c>
-      <c r="I15" s="1"/>
+      <c r="I15" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
@@ -963,7 +965,9 @@
       <c r="H16" s="1">
         <v>2203.8000000000002</v>
       </c>
-      <c r="I16" s="1"/>
+      <c r="I16" s="1">
+        <v>2782.9</v>
+      </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
@@ -986,7 +990,9 @@
       <c r="H17" s="1">
         <v>42.3</v>
       </c>
-      <c r="I17" s="1"/>
+      <c r="I17" s="1">
+        <v>51.3</v>
+      </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
@@ -1012,12 +1018,12 @@
         <v>0</v>
       </c>
       <c r="H18" s="1">
-        <f t="shared" ref="H18" si="7">H16-H17</f>
+        <f t="shared" ref="H18:I18" si="7">H16-H17</f>
         <v>2161.5</v>
       </c>
       <c r="I18" s="1">
-        <f t="shared" ref="I18" si="8">I16-I17</f>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>2731.6</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
@@ -1026,7 +1032,7 @@
       </c>
       <c r="B19" s="1">
         <f>SUM(E16:I16)/1000</f>
-        <v>6.2095000000000002</v>
+        <v>8.9923999999999999</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>8</v>
@@ -1041,7 +1047,9 @@
       <c r="H19" s="1">
         <v>81</v>
       </c>
-      <c r="I19" s="1"/>
+      <c r="I19" s="1">
+        <v>112</v>
+      </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
@@ -1049,7 +1057,7 @@
       </c>
       <c r="B20" s="1">
         <f>SUM(E19:I19)</f>
-        <v>231</v>
+        <v>343</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>9</v>
@@ -1064,7 +1072,9 @@
       <c r="H20" s="1">
         <v>31</v>
       </c>
-      <c r="I20" s="1"/>
+      <c r="I20" s="1">
+        <v>71</v>
+      </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
@@ -1072,7 +1082,7 @@
       </c>
       <c r="B21" s="1">
         <f>SUM(E20:I20)</f>
-        <v>95</v>
+        <v>166</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
@@ -1081,7 +1091,7 @@
       </c>
       <c r="B22" s="2">
         <f>(B20*300)+(B21*250)</f>
-        <v>93050</v>
+        <v>144400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Swapped emergency luminaires for building A ground floor
Had EU emergency luminaires, swapped for AS/NZ compliant luminaires. Updated documentation, DIALux, and excel
</commit_message>
<xml_diff>
--- a/Excel/Cost and CO2 analysis.xlsx
+++ b/Excel/Cost and CO2 analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester1\ELECTENG310\Alpha_Design_17\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13808E69-2BB3-4B5A-AD62-D9A4ABF80B23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{278D774E-F7EE-469A-BEE4-753D885F4CC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F8E8E83B-9F9C-423D-B7EA-650D4FA9D87D}"/>
   </bookViews>
@@ -614,11 +614,11 @@
       </c>
       <c r="C3" s="2">
         <f>($B$16*$B$14*0.25*A3)+$B$18</f>
-        <v>74326.065000000002</v>
+        <v>74306.759999999995</v>
       </c>
       <c r="D3" s="2">
         <f t="shared" ref="D3:D12" si="1">$B$22+($B$14*$B$19*0.25*A3)</f>
-        <v>98172.837499999994</v>
+        <v>98166.897500000006</v>
       </c>
       <c r="E3" s="3">
         <f t="shared" ref="E3:E12" si="2">0.25*A3*$B$14*$B$15</f>
@@ -626,11 +626,11 @@
       </c>
       <c r="F3" s="3">
         <f t="shared" ref="F3:F12" si="3">0.25*A3*$B$14*$B$16</f>
-        <v>5026.0649999999996</v>
+        <v>5006.76</v>
       </c>
       <c r="G3" s="3">
         <f t="shared" ref="G3:G12" si="4">0.25*A3*$B$14*$B$19</f>
-        <v>5122.8375000000005</v>
+        <v>5116.8975</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -643,11 +643,11 @@
       </c>
       <c r="C4" s="2">
         <f t="shared" ref="C4:C12" si="5">($B$16*$B$14*0.25*A4)+$B$18</f>
-        <v>79352.13</v>
+        <v>79313.52</v>
       </c>
       <c r="D4" s="2">
         <f t="shared" si="1"/>
-        <v>103295.675</v>
+        <v>103283.795</v>
       </c>
       <c r="E4" s="3">
         <f t="shared" si="2"/>
@@ -655,11 +655,11 @@
       </c>
       <c r="F4" s="3">
         <f t="shared" si="3"/>
-        <v>10052.129999999999</v>
+        <v>10013.52</v>
       </c>
       <c r="G4" s="3">
         <f t="shared" si="4"/>
-        <v>10245.675000000001</v>
+        <v>10233.795</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -672,11 +672,11 @@
       </c>
       <c r="C5" s="2">
         <f t="shared" si="5"/>
-        <v>84378.195000000007</v>
+        <v>84320.28</v>
       </c>
       <c r="D5" s="2">
         <f t="shared" si="1"/>
-        <v>108418.5125</v>
+        <v>108400.6925</v>
       </c>
       <c r="E5" s="3">
         <f t="shared" si="2"/>
@@ -684,11 +684,11 @@
       </c>
       <c r="F5" s="3">
         <f t="shared" si="3"/>
-        <v>15078.195</v>
+        <v>15020.28</v>
       </c>
       <c r="G5" s="3">
         <f t="shared" si="4"/>
-        <v>15368.512500000001</v>
+        <v>15350.692500000001</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -701,11 +701,11 @@
       </c>
       <c r="C6" s="2">
         <f t="shared" si="5"/>
-        <v>89404.26</v>
+        <v>89327.040000000008</v>
       </c>
       <c r="D6" s="2">
         <f t="shared" si="1"/>
-        <v>113541.35</v>
+        <v>113517.59</v>
       </c>
       <c r="E6" s="3">
         <f t="shared" si="2"/>
@@ -713,11 +713,11 @@
       </c>
       <c r="F6" s="3">
         <f t="shared" si="3"/>
-        <v>20104.259999999998</v>
+        <v>20027.04</v>
       </c>
       <c r="G6" s="3">
         <f t="shared" si="4"/>
-        <v>20491.350000000002</v>
+        <v>20467.59</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -730,11 +730,11 @@
       </c>
       <c r="C7" s="2">
         <f t="shared" si="5"/>
-        <v>94430.324999999997</v>
+        <v>94333.8</v>
       </c>
       <c r="D7" s="2">
         <f t="shared" si="1"/>
-        <v>118664.1875</v>
+        <v>118634.4875</v>
       </c>
       <c r="E7" s="3">
         <f t="shared" si="2"/>
@@ -742,11 +742,11 @@
       </c>
       <c r="F7" s="3">
         <f t="shared" si="3"/>
-        <v>25130.325000000001</v>
+        <v>25033.800000000003</v>
       </c>
       <c r="G7" s="3">
         <f t="shared" si="4"/>
-        <v>25614.1875</v>
+        <v>25584.487499999999</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -759,11 +759,11 @@
       </c>
       <c r="C8" s="2">
         <f t="shared" si="5"/>
-        <v>99456.39</v>
+        <v>99340.56</v>
       </c>
       <c r="D8" s="2">
         <f t="shared" si="1"/>
-        <v>123787.02499999999</v>
+        <v>123751.38500000001</v>
       </c>
       <c r="E8" s="3">
         <f t="shared" si="2"/>
@@ -771,11 +771,11 @@
       </c>
       <c r="F8" s="3">
         <f t="shared" si="3"/>
-        <v>30156.39</v>
+        <v>30040.560000000001</v>
       </c>
       <c r="G8" s="3">
         <f t="shared" si="4"/>
-        <v>30737.025000000001</v>
+        <v>30701.385000000002</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -788,11 +788,11 @@
       </c>
       <c r="C9" s="2">
         <f t="shared" si="5"/>
-        <v>104482.45499999999</v>
+        <v>104347.32</v>
       </c>
       <c r="D9" s="2">
         <f t="shared" si="1"/>
-        <v>128909.8625</v>
+        <v>128868.2825</v>
       </c>
       <c r="E9" s="3">
         <f t="shared" si="2"/>
@@ -800,11 +800,11 @@
       </c>
       <c r="F9" s="3">
         <f t="shared" si="3"/>
-        <v>35182.455000000002</v>
+        <v>35047.32</v>
       </c>
       <c r="G9" s="3">
         <f t="shared" si="4"/>
-        <v>35859.862500000003</v>
+        <v>35818.282500000001</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -817,11 +817,11 @@
       </c>
       <c r="C10" s="2">
         <f t="shared" si="5"/>
-        <v>109508.51999999999</v>
+        <v>109354.08</v>
       </c>
       <c r="D10" s="2">
         <f t="shared" si="1"/>
-        <v>134032.70000000001</v>
+        <v>133985.18</v>
       </c>
       <c r="E10" s="3">
         <f t="shared" si="2"/>
@@ -829,11 +829,11 @@
       </c>
       <c r="F10" s="3">
         <f t="shared" si="3"/>
-        <v>40208.519999999997</v>
+        <v>40054.080000000002</v>
       </c>
       <c r="G10" s="3">
         <f t="shared" si="4"/>
-        <v>40982.700000000004</v>
+        <v>40935.18</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -846,11 +846,11 @@
       </c>
       <c r="C11" s="2">
         <f t="shared" si="5"/>
-        <v>114534.58499999999</v>
+        <v>114360.84</v>
       </c>
       <c r="D11" s="2">
         <f t="shared" si="1"/>
-        <v>139155.53750000001</v>
+        <v>139102.07750000001</v>
       </c>
       <c r="E11" s="3">
         <f t="shared" si="2"/>
@@ -858,11 +858,11 @@
       </c>
       <c r="F11" s="3">
         <f t="shared" si="3"/>
-        <v>45234.584999999999</v>
+        <v>45060.840000000004</v>
       </c>
       <c r="G11" s="3">
         <f t="shared" si="4"/>
-        <v>46105.537499999999</v>
+        <v>46052.077499999999</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -875,11 +875,11 @@
       </c>
       <c r="C12" s="2">
         <f t="shared" si="5"/>
-        <v>119560.65</v>
+        <v>119367.6</v>
       </c>
       <c r="D12" s="2">
         <f t="shared" si="1"/>
-        <v>144278.375</v>
+        <v>144218.97500000001</v>
       </c>
       <c r="E12" s="3">
         <f t="shared" si="2"/>
@@ -887,11 +887,11 @@
       </c>
       <c r="F12" s="3">
         <f t="shared" si="3"/>
-        <v>50260.65</v>
+        <v>50067.600000000006</v>
       </c>
       <c r="G12" s="3">
         <f t="shared" si="4"/>
-        <v>51228.375</v>
+        <v>51168.974999999999</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
@@ -948,13 +948,13 @@
       </c>
       <c r="B16" s="1">
         <f>SUM(E18:H18)/1000</f>
-        <v>6.0922000000000001</v>
+        <v>6.0688000000000004</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E16" s="1">
-        <v>1100.7</v>
+        <v>1093.5</v>
       </c>
       <c r="F16" s="1">
         <v>2905</v>
@@ -977,7 +977,7 @@
         <v>25</v>
       </c>
       <c r="E17" s="1">
-        <v>30</v>
+        <v>46.2</v>
       </c>
       <c r="F17" s="1">
         <v>45</v>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="E18" s="1">
         <f>E16-E17</f>
-        <v>1070.7</v>
+        <v>1047.3</v>
       </c>
       <c r="F18" s="1">
         <f>F16-F17</f>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="B19" s="1">
         <f>SUM(E16:I16)/1000</f>
-        <v>6.2095000000000002</v>
+        <v>6.2023000000000001</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
Updated excel for building A ground floor
</commit_message>
<xml_diff>
--- a/Excel/Cost and CO2 analysis.xlsx
+++ b/Excel/Cost and CO2 analysis.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\310_Project1\Alpha_Design_17\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester1\ELECTENG310\Alpha_Design_17\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FE54094-97F6-4839-AA0B-E9AF3D2B7AAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA5FA7B-247A-443B-AB38-AF17296C5DA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F8E8E83B-9F9C-423D-B7EA-650D4FA9D87D}"/>
   </bookViews>
@@ -614,11 +614,11 @@
       </c>
       <c r="C3" s="2">
         <f>($B$16*$B$14*0.25*A3)+$B$18</f>
-        <v>74326.065000000002</v>
+        <v>74306.759999999995</v>
       </c>
       <c r="D3" s="2">
         <f t="shared" ref="D3:D12" si="1">$B$22+($B$14*$B$19*0.25*A3)</f>
-        <v>151818.73000000001</v>
+        <v>151812.79</v>
       </c>
       <c r="E3" s="3">
         <f t="shared" ref="E3:E12" si="2">0.25*A3*$B$14*$B$15</f>
@@ -626,11 +626,11 @@
       </c>
       <c r="F3" s="3">
         <f t="shared" ref="F3:F12" si="3">0.25*A3*$B$14*$B$16</f>
-        <v>5026.0649999999996</v>
+        <v>5006.76</v>
       </c>
       <c r="G3" s="3">
         <f t="shared" ref="G3:G12" si="4">0.25*A3*$B$14*$B$19</f>
-        <v>7418.73</v>
+        <v>7412.7900000000009</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -643,11 +643,11 @@
       </c>
       <c r="C4" s="2">
         <f t="shared" ref="C4:C12" si="5">($B$16*$B$14*0.25*A4)+$B$18</f>
-        <v>79352.13</v>
+        <v>79313.52</v>
       </c>
       <c r="D4" s="2">
         <f t="shared" si="1"/>
-        <v>159237.46</v>
+        <v>159225.58000000002</v>
       </c>
       <c r="E4" s="3">
         <f t="shared" si="2"/>
@@ -655,11 +655,11 @@
       </c>
       <c r="F4" s="3">
         <f t="shared" si="3"/>
-        <v>10052.129999999999</v>
+        <v>10013.52</v>
       </c>
       <c r="G4" s="3">
         <f t="shared" si="4"/>
-        <v>14837.46</v>
+        <v>14825.580000000002</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -672,11 +672,11 @@
       </c>
       <c r="C5" s="2">
         <f t="shared" si="5"/>
-        <v>84378.195000000007</v>
+        <v>84320.28</v>
       </c>
       <c r="D5" s="2">
         <f t="shared" si="1"/>
-        <v>166656.19</v>
+        <v>166638.37</v>
       </c>
       <c r="E5" s="3">
         <f t="shared" si="2"/>
@@ -684,11 +684,11 @@
       </c>
       <c r="F5" s="3">
         <f t="shared" si="3"/>
-        <v>15078.195</v>
+        <v>15020.28</v>
       </c>
       <c r="G5" s="3">
         <f t="shared" si="4"/>
-        <v>22256.19</v>
+        <v>22238.370000000003</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -701,11 +701,11 @@
       </c>
       <c r="C6" s="2">
         <f t="shared" si="5"/>
-        <v>89404.26</v>
+        <v>89327.040000000008</v>
       </c>
       <c r="D6" s="2">
         <f t="shared" si="1"/>
-        <v>174074.91999999998</v>
+        <v>174051.16</v>
       </c>
       <c r="E6" s="3">
         <f t="shared" si="2"/>
@@ -713,11 +713,11 @@
       </c>
       <c r="F6" s="3">
         <f t="shared" si="3"/>
-        <v>20104.259999999998</v>
+        <v>20027.04</v>
       </c>
       <c r="G6" s="3">
         <f t="shared" si="4"/>
-        <v>29674.92</v>
+        <v>29651.160000000003</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -730,11 +730,11 @@
       </c>
       <c r="C7" s="2">
         <f t="shared" si="5"/>
-        <v>94430.324999999997</v>
+        <v>94333.8</v>
       </c>
       <c r="D7" s="2">
         <f t="shared" si="1"/>
-        <v>181493.65</v>
+        <v>181463.95</v>
       </c>
       <c r="E7" s="3">
         <f t="shared" si="2"/>
@@ -742,11 +742,11 @@
       </c>
       <c r="F7" s="3">
         <f t="shared" si="3"/>
-        <v>25130.325000000001</v>
+        <v>25033.800000000003</v>
       </c>
       <c r="G7" s="3">
         <f t="shared" si="4"/>
-        <v>37093.65</v>
+        <v>37063.950000000004</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -759,11 +759,11 @@
       </c>
       <c r="C8" s="2">
         <f t="shared" si="5"/>
-        <v>99456.39</v>
+        <v>99340.56</v>
       </c>
       <c r="D8" s="2">
         <f t="shared" si="1"/>
-        <v>188912.38</v>
+        <v>188876.74</v>
       </c>
       <c r="E8" s="3">
         <f t="shared" si="2"/>
@@ -771,11 +771,11 @@
       </c>
       <c r="F8" s="3">
         <f t="shared" si="3"/>
-        <v>30156.39</v>
+        <v>30040.560000000001</v>
       </c>
       <c r="G8" s="3">
         <f t="shared" si="4"/>
-        <v>44512.38</v>
+        <v>44476.740000000005</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -788,11 +788,11 @@
       </c>
       <c r="C9" s="2">
         <f t="shared" si="5"/>
-        <v>104482.45499999999</v>
+        <v>104347.32</v>
       </c>
       <c r="D9" s="2">
         <f t="shared" si="1"/>
-        <v>196331.11</v>
+        <v>196289.53</v>
       </c>
       <c r="E9" s="3">
         <f t="shared" si="2"/>
@@ -800,11 +800,11 @@
       </c>
       <c r="F9" s="3">
         <f t="shared" si="3"/>
-        <v>35182.455000000002</v>
+        <v>35047.32</v>
       </c>
       <c r="G9" s="3">
         <f t="shared" si="4"/>
-        <v>51931.11</v>
+        <v>51889.530000000006</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -817,11 +817,11 @@
       </c>
       <c r="C10" s="2">
         <f t="shared" si="5"/>
-        <v>109508.51999999999</v>
+        <v>109354.08</v>
       </c>
       <c r="D10" s="2">
         <f t="shared" si="1"/>
-        <v>203749.84</v>
+        <v>203702.32</v>
       </c>
       <c r="E10" s="3">
         <f t="shared" si="2"/>
@@ -829,11 +829,11 @@
       </c>
       <c r="F10" s="3">
         <f t="shared" si="3"/>
-        <v>40208.519999999997</v>
+        <v>40054.080000000002</v>
       </c>
       <c r="G10" s="3">
         <f t="shared" si="4"/>
-        <v>59349.84</v>
+        <v>59302.320000000007</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -846,11 +846,11 @@
       </c>
       <c r="C11" s="2">
         <f t="shared" si="5"/>
-        <v>114534.58499999999</v>
+        <v>114360.84</v>
       </c>
       <c r="D11" s="2">
         <f t="shared" si="1"/>
-        <v>211168.57</v>
+        <v>211115.11000000002</v>
       </c>
       <c r="E11" s="3">
         <f t="shared" si="2"/>
@@ -858,11 +858,11 @@
       </c>
       <c r="F11" s="3">
         <f t="shared" si="3"/>
-        <v>45234.584999999999</v>
+        <v>45060.840000000004</v>
       </c>
       <c r="G11" s="3">
         <f t="shared" si="4"/>
-        <v>66768.569999999992</v>
+        <v>66715.11</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -875,11 +875,11 @@
       </c>
       <c r="C12" s="2">
         <f t="shared" si="5"/>
-        <v>119560.65</v>
+        <v>119367.6</v>
       </c>
       <c r="D12" s="2">
         <f t="shared" si="1"/>
-        <v>218587.3</v>
+        <v>218527.90000000002</v>
       </c>
       <c r="E12" s="3">
         <f t="shared" si="2"/>
@@ -887,11 +887,11 @@
       </c>
       <c r="F12" s="3">
         <f t="shared" si="3"/>
-        <v>50260.65</v>
+        <v>50067.600000000006</v>
       </c>
       <c r="G12" s="3">
         <f t="shared" si="4"/>
-        <v>74187.3</v>
+        <v>74127.900000000009</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
@@ -950,13 +950,13 @@
       </c>
       <c r="B16" s="1">
         <f>SUM(E18:H18)/1000</f>
-        <v>6.0922000000000001</v>
+        <v>6.0688000000000004</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E16" s="1">
-        <v>1100.7</v>
+        <v>1093.5</v>
       </c>
       <c r="F16" s="1">
         <v>2905</v>
@@ -981,7 +981,7 @@
         <v>25</v>
       </c>
       <c r="E17" s="1">
-        <v>30</v>
+        <v>46.2</v>
       </c>
       <c r="F17" s="1">
         <v>45</v>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E18" s="1">
         <f>E16-E17</f>
-        <v>1070.7</v>
+        <v>1047.3</v>
       </c>
       <c r="F18" s="1">
         <f>F16-F17</f>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="B19" s="1">
         <f>SUM(E16:I16)/1000</f>
-        <v>8.9923999999999999</v>
+        <v>8.9852000000000007</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
Optimised design to reduce cost.
</commit_message>
<xml_diff>
--- a/Excel/Cost and CO2 analysis.xlsx
+++ b/Excel/Cost and CO2 analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester1\ELECTENG310\Alpha_Design_17\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\Alpha_Design_17\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA5FA7B-247A-443B-AB38-AF17296C5DA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D08AE357-29A5-4178-881E-7D5D12B5F4BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F8E8E83B-9F9C-423D-B7EA-650D4FA9D87D}"/>
+    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F8E8E83B-9F9C-423D-B7EA-650D4FA9D87D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,9 +27,10 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -126,7 +127,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -214,6 +215,1279 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-NZ"/>
+              <a:t>Comparing</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-NZ" baseline="0"/>
+              <a:t> Existing and Proposed System Costs</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-NZ"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Existing System Cost ($)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$A$2:$A$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$B$2:$B$12</c:f>
+              <c:numCache>
+                <c:formatCode>_("$"* #,##0.00_);_("$"* \(#,##0.00\);_("$"* "-"??_);_(@_)</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>14556.3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>29112.6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>43668.899999999994</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>58225.2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>72781.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>87337.799999999988</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>101894.09999999999</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>116450.4</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>131006.7</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>145563</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-3327-4869-83B3-70829AA064EA}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Proposed System Cost ($)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$A$2:$A$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$C$2:$C$12</c:f>
+              <c:numCache>
+                <c:formatCode>_("$"* #,##0.00_);_("$"* \(#,##0.00\);_("$"* "-"??_);_(@_)</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>68400</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>73341.172500000001</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>78282.345000000001</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>83223.517500000002</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>88164.69</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>93105.862500000003</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>98047.035000000003</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>102988.20749999999</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>107929.38</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>112870.55249999999</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>117811.72500000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-3327-4869-83B3-70829AA064EA}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="553549344"/>
+        <c:axId val="553540192"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="553549344"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-NZ"/>
+                  <a:t>Years</a:t>
+                </a:r>
+              </a:p>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:endParaRPr lang="en-NZ"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="553540192"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="553540192"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-NZ"/>
+                  <a:t> Ttal</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-NZ" baseline="0"/>
+                  <a:t> Cost</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="553549344"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1030941</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>46704</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>49585</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0EC583EE-6DF1-45A6-9A7F-9CD2BD773BD9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -534,25 +1808,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD7E6F8D-4308-4D2A-878D-2A8D77E451CB}">
   <dimension ref="A1:I22"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="41.44140625" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" customWidth="1"/>
-    <col min="3" max="3" width="25.77734375" customWidth="1"/>
-    <col min="4" max="4" width="27.109375" customWidth="1"/>
-    <col min="5" max="5" width="29.44140625" customWidth="1"/>
-    <col min="6" max="6" width="29.33203125" customWidth="1"/>
-    <col min="7" max="7" width="19.109375" customWidth="1"/>
-    <col min="8" max="8" width="23.44140625" customWidth="1"/>
-    <col min="9" max="9" width="35.44140625" customWidth="1"/>
-    <col min="10" max="10" width="22.44140625" customWidth="1"/>
-    <col min="11" max="11" width="17.44140625" customWidth="1"/>
-    <col min="12" max="12" width="18.44140625" customWidth="1"/>
-    <col min="13" max="13" width="16.109375" customWidth="1"/>
-    <col min="14" max="14" width="19.44140625" customWidth="1"/>
+    <col min="1" max="1" width="41.4375" customWidth="1"/>
+    <col min="2" max="2" width="23.6875" customWidth="1"/>
+    <col min="3" max="3" width="25.75" customWidth="1"/>
+    <col min="4" max="4" width="27.125" customWidth="1"/>
+    <col min="5" max="5" width="29.4375" customWidth="1"/>
+    <col min="6" max="6" width="29.3125" customWidth="1"/>
+    <col min="7" max="7" width="19.125" customWidth="1"/>
+    <col min="8" max="8" width="23.4375" customWidth="1"/>
+    <col min="9" max="9" width="35.4375" customWidth="1"/>
+    <col min="10" max="10" width="22.4375" customWidth="1"/>
+    <col min="11" max="11" width="17.4375" customWidth="1"/>
+    <col min="12" max="12" width="18.4375" customWidth="1"/>
+    <col min="13" max="13" width="16.125" customWidth="1"/>
+    <col min="14" max="14" width="19.4375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="13.9">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -575,7 +1849,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="13.9">
       <c r="A2" s="4">
         <v>0</v>
       </c>
@@ -585,11 +1859,11 @@
       </c>
       <c r="C2" s="2">
         <f>($B$16*$B$14*0.25*A2)+$B$18</f>
-        <v>69300</v>
+        <v>68400</v>
       </c>
       <c r="D2" s="2">
         <f>$B$22+($B$14*$B$19*0.25*A2)</f>
-        <v>144400</v>
+        <v>143000</v>
       </c>
       <c r="E2" s="3">
         <f>0.25*A2*$B$14*$B$15</f>
@@ -604,7 +1878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="13.9">
       <c r="A3" s="4">
         <v>1</v>
       </c>
@@ -614,11 +1888,11 @@
       </c>
       <c r="C3" s="2">
         <f>($B$16*$B$14*0.25*A3)+$B$18</f>
-        <v>74306.759999999995</v>
+        <v>73341.172500000001</v>
       </c>
       <c r="D3" s="2">
         <f t="shared" ref="D3:D12" si="1">$B$22+($B$14*$B$19*0.25*A3)</f>
-        <v>151812.79</v>
+        <v>150345.7175</v>
       </c>
       <c r="E3" s="3">
         <f t="shared" ref="E3:E12" si="2">0.25*A3*$B$14*$B$15</f>
@@ -626,14 +1900,14 @@
       </c>
       <c r="F3" s="3">
         <f t="shared" ref="F3:F12" si="3">0.25*A3*$B$14*$B$16</f>
-        <v>5006.76</v>
+        <v>4941.1724999999997</v>
       </c>
       <c r="G3" s="3">
         <f t="shared" ref="G3:G12" si="4">0.25*A3*$B$14*$B$19</f>
-        <v>7412.7900000000009</v>
+        <v>7345.7174999999997</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="13.9">
       <c r="A4" s="4">
         <v>2</v>
       </c>
@@ -643,11 +1917,11 @@
       </c>
       <c r="C4" s="2">
         <f t="shared" ref="C4:C12" si="5">($B$16*$B$14*0.25*A4)+$B$18</f>
-        <v>79313.52</v>
+        <v>78282.345000000001</v>
       </c>
       <c r="D4" s="2">
         <f t="shared" si="1"/>
-        <v>159225.58000000002</v>
+        <v>157691.435</v>
       </c>
       <c r="E4" s="3">
         <f t="shared" si="2"/>
@@ -655,14 +1929,14 @@
       </c>
       <c r="F4" s="3">
         <f t="shared" si="3"/>
-        <v>10013.52</v>
+        <v>9882.3449999999993</v>
       </c>
       <c r="G4" s="3">
         <f t="shared" si="4"/>
-        <v>14825.580000000002</v>
+        <v>14691.434999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="13.9">
       <c r="A5" s="4">
         <v>3</v>
       </c>
@@ -672,11 +1946,11 @@
       </c>
       <c r="C5" s="2">
         <f t="shared" si="5"/>
-        <v>84320.28</v>
+        <v>83223.517500000002</v>
       </c>
       <c r="D5" s="2">
         <f t="shared" si="1"/>
-        <v>166638.37</v>
+        <v>165037.1525</v>
       </c>
       <c r="E5" s="3">
         <f t="shared" si="2"/>
@@ -684,14 +1958,14 @@
       </c>
       <c r="F5" s="3">
         <f t="shared" si="3"/>
-        <v>15020.28</v>
+        <v>14823.5175</v>
       </c>
       <c r="G5" s="3">
         <f t="shared" si="4"/>
-        <v>22238.370000000003</v>
+        <v>22037.1525</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="13.9">
       <c r="A6" s="4">
         <v>4</v>
       </c>
@@ -701,11 +1975,11 @@
       </c>
       <c r="C6" s="2">
         <f t="shared" si="5"/>
-        <v>89327.040000000008</v>
+        <v>88164.69</v>
       </c>
       <c r="D6" s="2">
         <f t="shared" si="1"/>
-        <v>174051.16</v>
+        <v>172382.87</v>
       </c>
       <c r="E6" s="3">
         <f t="shared" si="2"/>
@@ -713,14 +1987,14 @@
       </c>
       <c r="F6" s="3">
         <f t="shared" si="3"/>
-        <v>20027.04</v>
+        <v>19764.689999999999</v>
       </c>
       <c r="G6" s="3">
         <f t="shared" si="4"/>
-        <v>29651.160000000003</v>
+        <v>29382.87</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="13.9">
       <c r="A7" s="4">
         <v>5</v>
       </c>
@@ -730,11 +2004,11 @@
       </c>
       <c r="C7" s="2">
         <f t="shared" si="5"/>
-        <v>94333.8</v>
+        <v>93105.862500000003</v>
       </c>
       <c r="D7" s="2">
         <f t="shared" si="1"/>
-        <v>181463.95</v>
+        <v>179728.58749999999</v>
       </c>
       <c r="E7" s="3">
         <f t="shared" si="2"/>
@@ -742,14 +2016,14 @@
       </c>
       <c r="F7" s="3">
         <f t="shared" si="3"/>
-        <v>25033.800000000003</v>
+        <v>24705.862499999999</v>
       </c>
       <c r="G7" s="3">
         <f t="shared" si="4"/>
-        <v>37063.950000000004</v>
+        <v>36728.587500000001</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="13.9">
       <c r="A8" s="4">
         <v>6</v>
       </c>
@@ -759,11 +2033,11 @@
       </c>
       <c r="C8" s="2">
         <f t="shared" si="5"/>
-        <v>99340.56</v>
+        <v>98047.035000000003</v>
       </c>
       <c r="D8" s="2">
         <f t="shared" si="1"/>
-        <v>188876.74</v>
+        <v>187074.30499999999</v>
       </c>
       <c r="E8" s="3">
         <f t="shared" si="2"/>
@@ -771,14 +2045,14 @@
       </c>
       <c r="F8" s="3">
         <f t="shared" si="3"/>
-        <v>30040.560000000001</v>
+        <v>29647.035</v>
       </c>
       <c r="G8" s="3">
         <f t="shared" si="4"/>
-        <v>44476.740000000005</v>
+        <v>44074.305</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="13.9">
       <c r="A9" s="4">
         <v>7</v>
       </c>
@@ -788,11 +2062,11 @@
       </c>
       <c r="C9" s="2">
         <f t="shared" si="5"/>
-        <v>104347.32</v>
+        <v>102988.20749999999</v>
       </c>
       <c r="D9" s="2">
         <f t="shared" si="1"/>
-        <v>196289.53</v>
+        <v>194420.02249999999</v>
       </c>
       <c r="E9" s="3">
         <f t="shared" si="2"/>
@@ -800,14 +2074,14 @@
       </c>
       <c r="F9" s="3">
         <f t="shared" si="3"/>
-        <v>35047.32</v>
+        <v>34588.207499999997</v>
       </c>
       <c r="G9" s="3">
         <f t="shared" si="4"/>
-        <v>51889.530000000006</v>
+        <v>51420.022499999999</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="13.9">
       <c r="A10" s="4">
         <v>8</v>
       </c>
@@ -817,11 +2091,11 @@
       </c>
       <c r="C10" s="2">
         <f t="shared" si="5"/>
-        <v>109354.08</v>
+        <v>107929.38</v>
       </c>
       <c r="D10" s="2">
         <f t="shared" si="1"/>
-        <v>203702.32</v>
+        <v>201765.74</v>
       </c>
       <c r="E10" s="3">
         <f t="shared" si="2"/>
@@ -829,14 +2103,14 @@
       </c>
       <c r="F10" s="3">
         <f t="shared" si="3"/>
-        <v>40054.080000000002</v>
+        <v>39529.379999999997</v>
       </c>
       <c r="G10" s="3">
         <f t="shared" si="4"/>
-        <v>59302.320000000007</v>
+        <v>58765.74</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="13.9">
       <c r="A11" s="4">
         <v>9</v>
       </c>
@@ -846,11 +2120,11 @@
       </c>
       <c r="C11" s="2">
         <f t="shared" si="5"/>
-        <v>114360.84</v>
+        <v>112870.55249999999</v>
       </c>
       <c r="D11" s="2">
         <f t="shared" si="1"/>
-        <v>211115.11000000002</v>
+        <v>209111.45750000002</v>
       </c>
       <c r="E11" s="3">
         <f t="shared" si="2"/>
@@ -858,14 +2132,14 @@
       </c>
       <c r="F11" s="3">
         <f t="shared" si="3"/>
-        <v>45060.840000000004</v>
+        <v>44470.552499999998</v>
       </c>
       <c r="G11" s="3">
         <f t="shared" si="4"/>
-        <v>66715.11</v>
+        <v>66111.457500000004</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="13.9">
       <c r="A12" s="4">
         <v>10</v>
       </c>
@@ -875,11 +2149,11 @@
       </c>
       <c r="C12" s="2">
         <f t="shared" si="5"/>
-        <v>119367.6</v>
+        <v>117811.72500000001</v>
       </c>
       <c r="D12" s="2">
         <f t="shared" si="1"/>
-        <v>218527.90000000002</v>
+        <v>216457.17499999999</v>
       </c>
       <c r="E12" s="3">
         <f t="shared" si="2"/>
@@ -887,14 +2161,14 @@
       </c>
       <c r="F12" s="3">
         <f t="shared" si="3"/>
-        <v>50067.600000000006</v>
+        <v>49411.724999999999</v>
       </c>
       <c r="G12" s="3">
         <f t="shared" si="4"/>
-        <v>74127.900000000009</v>
+        <v>73457.175000000003</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="13.9">
       <c r="A14" s="4" t="s">
         <v>1</v>
       </c>
@@ -919,7 +2193,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="13.9">
       <c r="A15" s="4" t="s">
         <v>12</v>
       </c>
@@ -944,13 +2218,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="13.9">
       <c r="A16" s="4" t="s">
         <v>11</v>
       </c>
       <c r="B16" s="1">
         <f>SUM(E18:H18)/1000</f>
-        <v>6.0688000000000004</v>
+        <v>5.9893000000000001</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>24</v>
@@ -963,19 +2237,19 @@
       </c>
       <c r="G16" s="1"/>
       <c r="H16" s="1">
-        <v>2203.8000000000002</v>
+        <v>2122.5</v>
       </c>
       <c r="I16" s="1">
         <v>2782.9</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" ht="13.9">
       <c r="A17" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B17" s="3">
         <f>SUM(E19:H19)</f>
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>25</v>
@@ -988,19 +2262,19 @@
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1">
-        <v>42.3</v>
+        <v>40.5</v>
       </c>
       <c r="I17" s="1">
         <v>51.3</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" ht="13.9">
       <c r="A18" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B18" s="2">
         <f>B17*300</f>
-        <v>69300</v>
+        <v>68400</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>26</v>
@@ -1019,20 +2293,20 @@
       </c>
       <c r="H18" s="1">
         <f t="shared" ref="H18:I18" si="7">H16-H17</f>
-        <v>2161.5</v>
+        <v>2082</v>
       </c>
       <c r="I18" s="1">
         <f t="shared" si="7"/>
         <v>2731.6</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" ht="13.9">
       <c r="A19" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B19" s="1">
         <f>SUM(E16:I16)/1000</f>
-        <v>8.9852000000000007</v>
+        <v>8.9039000000000001</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>8</v>
@@ -1045,19 +2319,19 @@
       </c>
       <c r="G19" s="1"/>
       <c r="H19" s="1">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="I19" s="1">
         <v>112</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" ht="13.9">
       <c r="A20" s="4" t="s">
         <v>16</v>
       </c>
       <c r="B20" s="1">
         <f>SUM(E19:I19)</f>
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>9</v>
@@ -1070,32 +2344,33 @@
       </c>
       <c r="G20" s="1"/>
       <c r="H20" s="1">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I20" s="1">
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="13.9">
       <c r="A21" s="4" t="s">
         <v>15</v>
       </c>
       <c r="B21" s="1">
         <f>SUM(E20:I20)</f>
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="13.9">
       <c r="A22" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B22" s="2">
         <f>(B20*300)+(B21*250)</f>
-        <v>144400</v>
+        <v>143000</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Added power use (4 W) for the two outdoor emergency luminaires for building A ground floor
</commit_message>
<xml_diff>
--- a/Excel/Cost and CO2 analysis.xlsx
+++ b/Excel/Cost and CO2 analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\Alpha_Design_17\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester1\ELECTENG310\Alpha_Design_17\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D08AE357-29A5-4178-881E-7D5D12B5F4BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E5BC5B6-54D2-460D-A3FB-2E4D7136E9B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F8E8E83B-9F9C-423D-B7EA-650D4FA9D87D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F8E8E83B-9F9C-423D-B7EA-650D4FA9D87D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,9 +29,6 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -127,7 +124,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -220,7 +217,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -287,7 +284,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-NZ"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -851,6 +848,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -858,7 +856,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1808,25 +1805,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD7E6F8D-4308-4D2A-878D-2A8D77E451CB}">
   <dimension ref="A1:I22"/>
-  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="41.4375" customWidth="1"/>
-    <col min="2" max="2" width="23.6875" customWidth="1"/>
-    <col min="3" max="3" width="25.75" customWidth="1"/>
-    <col min="4" max="4" width="27.125" customWidth="1"/>
-    <col min="5" max="5" width="29.4375" customWidth="1"/>
-    <col min="6" max="6" width="29.3125" customWidth="1"/>
-    <col min="7" max="7" width="19.125" customWidth="1"/>
-    <col min="8" max="8" width="23.4375" customWidth="1"/>
-    <col min="9" max="9" width="35.4375" customWidth="1"/>
-    <col min="10" max="10" width="22.4375" customWidth="1"/>
-    <col min="11" max="11" width="17.4375" customWidth="1"/>
-    <col min="12" max="12" width="18.4375" customWidth="1"/>
-    <col min="13" max="13" width="16.125" customWidth="1"/>
-    <col min="14" max="14" width="19.4375" customWidth="1"/>
+    <col min="1" max="1" width="41.44140625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" customWidth="1"/>
+    <col min="3" max="3" width="25.77734375" customWidth="1"/>
+    <col min="4" max="4" width="27.109375" customWidth="1"/>
+    <col min="5" max="5" width="29.44140625" customWidth="1"/>
+    <col min="6" max="6" width="29.33203125" customWidth="1"/>
+    <col min="7" max="7" width="19.109375" customWidth="1"/>
+    <col min="8" max="8" width="23.44140625" customWidth="1"/>
+    <col min="9" max="9" width="35.44140625" customWidth="1"/>
+    <col min="10" max="10" width="22.44140625" customWidth="1"/>
+    <col min="11" max="11" width="17.44140625" customWidth="1"/>
+    <col min="12" max="12" width="18.44140625" customWidth="1"/>
+    <col min="13" max="13" width="16.109375" customWidth="1"/>
+    <col min="14" max="14" width="19.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="13.9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1849,7 +1846,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="13.9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>0</v>
       </c>
@@ -1878,7 +1875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="13.9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>1</v>
       </c>
@@ -1892,7 +1889,7 @@
       </c>
       <c r="D3" s="2">
         <f t="shared" ref="D3:D12" si="1">$B$22+($B$14*$B$19*0.25*A3)</f>
-        <v>150345.7175</v>
+        <v>150349.01749999999</v>
       </c>
       <c r="E3" s="3">
         <f t="shared" ref="E3:E12" si="2">0.25*A3*$B$14*$B$15</f>
@@ -1904,10 +1901,10 @@
       </c>
       <c r="G3" s="3">
         <f t="shared" ref="G3:G12" si="4">0.25*A3*$B$14*$B$19</f>
-        <v>7345.7174999999997</v>
+        <v>7349.0174999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="13.9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>2</v>
       </c>
@@ -1921,7 +1918,7 @@
       </c>
       <c r="D4" s="2">
         <f t="shared" si="1"/>
-        <v>157691.435</v>
+        <v>157698.035</v>
       </c>
       <c r="E4" s="3">
         <f t="shared" si="2"/>
@@ -1933,10 +1930,10 @@
       </c>
       <c r="G4" s="3">
         <f t="shared" si="4"/>
-        <v>14691.434999999999</v>
+        <v>14698.035</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="13.9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>3</v>
       </c>
@@ -1950,7 +1947,7 @@
       </c>
       <c r="D5" s="2">
         <f t="shared" si="1"/>
-        <v>165037.1525</v>
+        <v>165047.05249999999</v>
       </c>
       <c r="E5" s="3">
         <f t="shared" si="2"/>
@@ -1962,10 +1959,10 @@
       </c>
       <c r="G5" s="3">
         <f t="shared" si="4"/>
-        <v>22037.1525</v>
+        <v>22047.052499999998</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="13.9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>4</v>
       </c>
@@ -1979,7 +1976,7 @@
       </c>
       <c r="D6" s="2">
         <f t="shared" si="1"/>
-        <v>172382.87</v>
+        <v>172396.07</v>
       </c>
       <c r="E6" s="3">
         <f t="shared" si="2"/>
@@ -1991,10 +1988,10 @@
       </c>
       <c r="G6" s="3">
         <f t="shared" si="4"/>
-        <v>29382.87</v>
+        <v>29396.07</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="13.9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>5</v>
       </c>
@@ -2008,7 +2005,7 @@
       </c>
       <c r="D7" s="2">
         <f t="shared" si="1"/>
-        <v>179728.58749999999</v>
+        <v>179745.08749999999</v>
       </c>
       <c r="E7" s="3">
         <f t="shared" si="2"/>
@@ -2020,10 +2017,10 @@
       </c>
       <c r="G7" s="3">
         <f t="shared" si="4"/>
-        <v>36728.587500000001</v>
+        <v>36745.087500000001</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="13.9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>6</v>
       </c>
@@ -2037,7 +2034,7 @@
       </c>
       <c r="D8" s="2">
         <f t="shared" si="1"/>
-        <v>187074.30499999999</v>
+        <v>187094.10499999998</v>
       </c>
       <c r="E8" s="3">
         <f t="shared" si="2"/>
@@ -2049,10 +2046,10 @@
       </c>
       <c r="G8" s="3">
         <f t="shared" si="4"/>
-        <v>44074.305</v>
+        <v>44094.104999999996</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="13.9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>7</v>
       </c>
@@ -2066,7 +2063,7 @@
       </c>
       <c r="D9" s="2">
         <f t="shared" si="1"/>
-        <v>194420.02249999999</v>
+        <v>194443.1225</v>
       </c>
       <c r="E9" s="3">
         <f t="shared" si="2"/>
@@ -2078,10 +2075,10 @@
       </c>
       <c r="G9" s="3">
         <f t="shared" si="4"/>
-        <v>51420.022499999999</v>
+        <v>51443.122499999998</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="13.9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>8</v>
       </c>
@@ -2095,7 +2092,7 @@
       </c>
       <c r="D10" s="2">
         <f t="shared" si="1"/>
-        <v>201765.74</v>
+        <v>201792.14</v>
       </c>
       <c r="E10" s="3">
         <f t="shared" si="2"/>
@@ -2107,10 +2104,10 @@
       </c>
       <c r="G10" s="3">
         <f t="shared" si="4"/>
-        <v>58765.74</v>
+        <v>58792.14</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="13.9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>9</v>
       </c>
@@ -2124,7 +2121,7 @@
       </c>
       <c r="D11" s="2">
         <f t="shared" si="1"/>
-        <v>209111.45750000002</v>
+        <v>209141.1575</v>
       </c>
       <c r="E11" s="3">
         <f t="shared" si="2"/>
@@ -2136,10 +2133,10 @@
       </c>
       <c r="G11" s="3">
         <f t="shared" si="4"/>
-        <v>66111.457500000004</v>
+        <v>66141.157500000001</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="13.9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>10</v>
       </c>
@@ -2153,7 +2150,7 @@
       </c>
       <c r="D12" s="2">
         <f t="shared" si="1"/>
-        <v>216457.17499999999</v>
+        <v>216490.17499999999</v>
       </c>
       <c r="E12" s="3">
         <f t="shared" si="2"/>
@@ -2165,10 +2162,10 @@
       </c>
       <c r="G12" s="3">
         <f t="shared" si="4"/>
-        <v>73457.175000000003</v>
+        <v>73490.175000000003</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="13.9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>1</v>
       </c>
@@ -2193,7 +2190,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="13.9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>12</v>
       </c>
@@ -2218,7 +2215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="13.9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>11</v>
       </c>
@@ -2230,7 +2227,7 @@
         <v>24</v>
       </c>
       <c r="E16" s="1">
-        <v>1093.5</v>
+        <v>1097.5</v>
       </c>
       <c r="F16" s="1">
         <v>2905</v>
@@ -2243,7 +2240,7 @@
         <v>2782.9</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="13.9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>10</v>
       </c>
@@ -2255,7 +2252,7 @@
         <v>25</v>
       </c>
       <c r="E17" s="1">
-        <v>46.2</v>
+        <v>50.2</v>
       </c>
       <c r="F17" s="1">
         <v>45</v>
@@ -2268,7 +2265,7 @@
         <v>51.3</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="13.9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>14</v>
       </c>
@@ -2300,13 +2297,13 @@
         <v>2731.6</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="13.9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B19" s="1">
         <f>SUM(E16:I16)/1000</f>
-        <v>8.9039000000000001</v>
+        <v>8.9078999999999997</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>8</v>
@@ -2325,7 +2322,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="13.9">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>16</v>
       </c>
@@ -2350,7 +2347,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="13.9">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>15</v>
       </c>
@@ -2359,7 +2356,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="13.9">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Updated report and excel.
</commit_message>
<xml_diff>
--- a/Excel/Cost and CO2 analysis.xlsx
+++ b/Excel/Cost and CO2 analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester1\ELECTENG310\Alpha_Design_17\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\Alpha_Design_17\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E5BC5B6-54D2-460D-A3FB-2E4D7136E9B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2F04172-5AE4-41D6-ACA1-8B77A760454A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F8E8E83B-9F9C-423D-B7EA-650D4FA9D87D}"/>
+    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F8E8E83B-9F9C-423D-B7EA-650D4FA9D87D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,12 +29,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Years</t>
   </si>
@@ -115,6 +118,12 @@
   </si>
   <si>
     <t>Power excl. emergency (W)</t>
+  </si>
+  <si>
+    <t>Hours per year (Carpark):</t>
+  </si>
+  <si>
+    <t>Total Power (excl. carpark) [kW]:</t>
   </si>
 </sst>
 </file>
@@ -124,7 +133,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -217,7 +226,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -284,7 +293,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-NZ"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -848,7 +857,6 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -856,6 +864,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1804,26 +1813,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD7E6F8D-4308-4D2A-878D-2A8D77E451CB}">
-  <dimension ref="A1:I22"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I24"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="41.44140625" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" customWidth="1"/>
-    <col min="3" max="3" width="25.77734375" customWidth="1"/>
-    <col min="4" max="4" width="27.109375" customWidth="1"/>
-    <col min="5" max="5" width="29.44140625" customWidth="1"/>
-    <col min="6" max="6" width="29.33203125" customWidth="1"/>
-    <col min="7" max="7" width="19.109375" customWidth="1"/>
-    <col min="8" max="8" width="23.44140625" customWidth="1"/>
-    <col min="9" max="9" width="35.44140625" customWidth="1"/>
-    <col min="10" max="10" width="22.44140625" customWidth="1"/>
-    <col min="11" max="11" width="17.44140625" customWidth="1"/>
-    <col min="12" max="12" width="18.44140625" customWidth="1"/>
-    <col min="13" max="13" width="16.109375" customWidth="1"/>
-    <col min="14" max="14" width="19.44140625" customWidth="1"/>
+    <col min="1" max="1" width="41.4375" customWidth="1"/>
+    <col min="2" max="2" width="23.6875" customWidth="1"/>
+    <col min="3" max="3" width="25.75" customWidth="1"/>
+    <col min="4" max="4" width="27.125" customWidth="1"/>
+    <col min="5" max="5" width="29.4375" customWidth="1"/>
+    <col min="6" max="6" width="29.3125" customWidth="1"/>
+    <col min="7" max="7" width="19.125" customWidth="1"/>
+    <col min="8" max="8" width="23.4375" customWidth="1"/>
+    <col min="9" max="9" width="35.4375" customWidth="1"/>
+    <col min="10" max="10" width="22.4375" customWidth="1"/>
+    <col min="11" max="11" width="17.4375" customWidth="1"/>
+    <col min="12" max="12" width="18.4375" customWidth="1"/>
+    <col min="13" max="13" width="16.125" customWidth="1"/>
+    <col min="14" max="14" width="19.4375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="13.9">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1846,7 +1855,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="13.9">
       <c r="A2" s="4">
         <v>0</v>
       </c>
@@ -1859,7 +1868,7 @@
         <v>68400</v>
       </c>
       <c r="D2" s="2">
-        <f>$B$22+($B$14*$B$19*0.25*A2)</f>
+        <f>$B$22+((($B$14*$B$24) + ($I$16*$B$23/1000)) *0.25*A2)</f>
         <v>143000</v>
       </c>
       <c r="E2" s="3">
@@ -1871,11 +1880,11 @@
         <v>0</v>
       </c>
       <c r="G2" s="3">
-        <f>0.25*A2*$B$14*$B$19</f>
+        <f>0.25*A2*(($B$14*$B$24)+($I$16*$B$23/1000))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="13.9">
       <c r="A3" s="4">
         <v>1</v>
       </c>
@@ -1888,8 +1897,8 @@
         <v>73341.172500000001</v>
       </c>
       <c r="D3" s="2">
-        <f t="shared" ref="D3:D12" si="1">$B$22+($B$14*$B$19*0.25*A3)</f>
-        <v>150349.01749999999</v>
+        <f t="shared" ref="D3:D12" si="1">$B$22+((($B$14*$B$24) + ($I$16*$B$23/1000)) *0.25*A3)</f>
+        <v>154130.9786</v>
       </c>
       <c r="E3" s="3">
         <f t="shared" ref="E3:E12" si="2">0.25*A3*$B$14*$B$15</f>
@@ -1900,11 +1909,11 @@
         <v>4941.1724999999997</v>
       </c>
       <c r="G3" s="3">
-        <f t="shared" ref="G3:G12" si="4">0.25*A3*$B$14*$B$19</f>
-        <v>7349.0174999999999</v>
+        <f t="shared" ref="G3:G12" si="4">0.25*A3*(($B$14*$B$24)+($I$16*$B$23/1000))</f>
+        <v>11130.9786</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="13.9">
       <c r="A4" s="4">
         <v>2</v>
       </c>
@@ -1918,7 +1927,7 @@
       </c>
       <c r="D4" s="2">
         <f t="shared" si="1"/>
-        <v>157698.035</v>
+        <v>165261.9572</v>
       </c>
       <c r="E4" s="3">
         <f t="shared" si="2"/>
@@ -1930,10 +1939,10 @@
       </c>
       <c r="G4" s="3">
         <f t="shared" si="4"/>
-        <v>14698.035</v>
+        <v>22261.957200000001</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="13.9">
       <c r="A5" s="4">
         <v>3</v>
       </c>
@@ -1947,7 +1956,7 @@
       </c>
       <c r="D5" s="2">
         <f t="shared" si="1"/>
-        <v>165047.05249999999</v>
+        <v>176392.93580000001</v>
       </c>
       <c r="E5" s="3">
         <f t="shared" si="2"/>
@@ -1959,10 +1968,10 @@
       </c>
       <c r="G5" s="3">
         <f t="shared" si="4"/>
-        <v>22047.052499999998</v>
+        <v>33392.935799999999</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="13.9">
       <c r="A6" s="4">
         <v>4</v>
       </c>
@@ -1976,7 +1985,7 @@
       </c>
       <c r="D6" s="2">
         <f t="shared" si="1"/>
-        <v>172396.07</v>
+        <v>187523.91440000001</v>
       </c>
       <c r="E6" s="3">
         <f t="shared" si="2"/>
@@ -1988,10 +1997,10 @@
       </c>
       <c r="G6" s="3">
         <f t="shared" si="4"/>
-        <v>29396.07</v>
+        <v>44523.914400000001</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="13.9">
       <c r="A7" s="4">
         <v>5</v>
       </c>
@@ -2005,7 +2014,7 @@
       </c>
       <c r="D7" s="2">
         <f t="shared" si="1"/>
-        <v>179745.08749999999</v>
+        <v>198654.89300000001</v>
       </c>
       <c r="E7" s="3">
         <f t="shared" si="2"/>
@@ -2017,10 +2026,10 @@
       </c>
       <c r="G7" s="3">
         <f t="shared" si="4"/>
-        <v>36745.087500000001</v>
+        <v>55654.893000000004</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="13.9">
       <c r="A8" s="4">
         <v>6</v>
       </c>
@@ -2034,7 +2043,7 @@
       </c>
       <c r="D8" s="2">
         <f t="shared" si="1"/>
-        <v>187094.10499999998</v>
+        <v>209785.87160000001</v>
       </c>
       <c r="E8" s="3">
         <f t="shared" si="2"/>
@@ -2046,10 +2055,10 @@
       </c>
       <c r="G8" s="3">
         <f t="shared" si="4"/>
-        <v>44094.104999999996</v>
+        <v>66785.871599999999</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="13.9">
       <c r="A9" s="4">
         <v>7</v>
       </c>
@@ -2063,7 +2072,7 @@
       </c>
       <c r="D9" s="2">
         <f t="shared" si="1"/>
-        <v>194443.1225</v>
+        <v>220916.85019999999</v>
       </c>
       <c r="E9" s="3">
         <f t="shared" si="2"/>
@@ -2075,10 +2084,10 @@
       </c>
       <c r="G9" s="3">
         <f t="shared" si="4"/>
-        <v>51443.122499999998</v>
+        <v>77916.850200000001</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="13.9">
       <c r="A10" s="4">
         <v>8</v>
       </c>
@@ -2092,7 +2101,7 @@
       </c>
       <c r="D10" s="2">
         <f t="shared" si="1"/>
-        <v>201792.14</v>
+        <v>232047.82880000002</v>
       </c>
       <c r="E10" s="3">
         <f t="shared" si="2"/>
@@ -2103,11 +2112,11 @@
         <v>39529.379999999997</v>
       </c>
       <c r="G10" s="3">
-        <f t="shared" si="4"/>
-        <v>58792.14</v>
+        <f>0.25*A10*(($B$14*$B$24)+($I$16*$B$23/1000))</f>
+        <v>89047.828800000003</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="13.9">
       <c r="A11" s="4">
         <v>9</v>
       </c>
@@ -2121,7 +2130,7 @@
       </c>
       <c r="D11" s="2">
         <f t="shared" si="1"/>
-        <v>209141.1575</v>
+        <v>243178.80739999999</v>
       </c>
       <c r="E11" s="3">
         <f t="shared" si="2"/>
@@ -2133,10 +2142,10 @@
       </c>
       <c r="G11" s="3">
         <f t="shared" si="4"/>
-        <v>66141.157500000001</v>
+        <v>100178.80740000001</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="13.9">
       <c r="A12" s="4">
         <v>10</v>
       </c>
@@ -2150,7 +2159,7 @@
       </c>
       <c r="D12" s="2">
         <f t="shared" si="1"/>
-        <v>216490.17499999999</v>
+        <v>254309.78600000002</v>
       </c>
       <c r="E12" s="3">
         <f t="shared" si="2"/>
@@ -2162,10 +2171,10 @@
       </c>
       <c r="G12" s="3">
         <f t="shared" si="4"/>
-        <v>73490.175000000003</v>
+        <v>111309.78600000001</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="13.9">
       <c r="A14" s="4" t="s">
         <v>1</v>
       </c>
@@ -2190,7 +2199,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="13.9">
       <c r="A15" s="4" t="s">
         <v>12</v>
       </c>
@@ -2215,7 +2224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="13.9">
       <c r="A16" s="4" t="s">
         <v>11</v>
       </c>
@@ -2240,7 +2249,7 @@
         <v>2782.9</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" ht="13.9">
       <c r="A17" s="4" t="s">
         <v>10</v>
       </c>
@@ -2265,7 +2274,7 @@
         <v>51.3</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" ht="13.9">
       <c r="A18" s="4" t="s">
         <v>14</v>
       </c>
@@ -2297,7 +2306,7 @@
         <v>2731.6</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" ht="13.9">
       <c r="A19" s="4" t="s">
         <v>13</v>
       </c>
@@ -2322,7 +2331,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" ht="13.9">
       <c r="A20" s="4" t="s">
         <v>16</v>
       </c>
@@ -2347,7 +2356,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="13.9">
       <c r="A21" s="4" t="s">
         <v>15</v>
       </c>
@@ -2356,13 +2365,31 @@
         <v>164</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="13.9">
       <c r="A22" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B22" s="2">
         <f>(B20*300)+(B21*250)</f>
         <v>143000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="13.9">
+      <c r="A23" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" s="1">
+        <f>24*52*7</f>
+        <v>8736</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="13.9">
+      <c r="A24" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" s="1">
+        <f>SUM(E16:H16)/1000</f>
+        <v>6.125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated report. Adjusted calculation planes and wall luminaire.
</commit_message>
<xml_diff>
--- a/Excel/Cost and CO2 analysis.xlsx
+++ b/Excel/Cost and CO2 analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\Alpha_Design_17\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4A10F68-4F54-4D16-A736-A8EA126E47E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{836F03A4-3429-4916-8BC9-5BBECCCB95BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F8E8E83B-9F9C-423D-B7EA-650D4FA9D87D}"/>
   </bookViews>
@@ -130,7 +130,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="3">
@@ -199,12 +200,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1813,7 +1815,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD7E6F8D-4308-4D2A-878D-2A8D77E451CB}">
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="41.4375" customWidth="1"/>
@@ -2401,6 +2403,19 @@
         <f>SUM(E16:H16)/1000</f>
         <v>7.8224999999999998</v>
       </c>
+      <c r="D24" s="5"/>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="D25" s="5"/>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="C26" s="5"/>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="C28">
+        <f>((SUM(E18:H18)*3300/1000)+(I18*8736/1000))*0.25</f>
+        <v>12260.811900000001</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>